<commit_message>
Settle Jul 30-31, demote Polymarket per ledger, ship Aug 1 all-markets card
Jul 30 fully settled (8/8; Brier ours .210 vs close .199 on the day) and
Jul 31 partially: both limit orders confirmed no-fill (the Pirates target
would have been ~+11% vs the close - right side, price never came) and
the NYY@CHC refusal validated (close landed on the book consensus;
Polymarket was the stale outlier again). Third documented 5-6pt Polymarket
miss -> sharpness demoted 0.65 to 0.45, below the anchor gate. Aug 1
slate adds the first priced totals market; card: pass, top order Reds ML
at >= 2.262, refusals on NYY@CHC (day 2), DET@ATH, WSH@ATL. Tracker
grade filter now skips refused markets (no prediction to grade).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Epz958ydWx4TMSQvnKeiSm
</commit_message>
<xml_diff>
--- a/data/tracker.xlsx
+++ b/data/tracker.xlsx
@@ -511,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:N15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -902,7 +902,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>validated</t>
         </is>
       </c>
       <c r="I7" s="5" t="n">
@@ -917,12 +917,12 @@
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>worked</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>Consensus CHC -142 vs Polymarket 52c -&gt; -2.17% pseudo-arb: yesterday's failure signature; refused under the new rule.</t>
+          <t>Close CHC -140 landed on the sportsbook consensus; Polymarket 52c was the stale outlier (NYY won 2-0 as a +130 dog - vs the close that bet was -7% EV luck). Refusal correct.</t>
         </is>
       </c>
     </row>
@@ -956,7 +956,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>no fill</t>
         </is>
       </c>
       <c r="I8" s="5" t="n">
@@ -971,12 +971,12 @@
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>worked</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>Listed 2.041 sits at fair (-0.2% EV); order rests at 2.10 where the SportsGrid Phillies lean is paid for.</t>
+          <t>PHI never traded above 2.06 (target 2.10). Close no-vig PHI 0.467: even at target the bet was -2% vs close - not filling saved money. SportsGrid model lean (PHI 54%) was the wrong side per the close.</t>
         </is>
       </c>
     </row>
@@ -1010,7 +1010,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>no fill</t>
         </is>
       </c>
       <c r="I9" s="5" t="n">
@@ -1025,17 +1025,229 @@
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
+          <t>worked</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>PIT -120 to -136 all day, never near the 1.966 target. Close no-vig PIT 0.564: a 1.966 fill would have been ~+11% EV vs close - right side, market never paid the price.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>PIT @ CIN</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Reds ML</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>order_open</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>2.262</v>
+      </c>
+      <c r="F10" s="3" t="n"/>
+      <c r="G10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
           <t>pending</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
-        <is>
-          <t>Runner-up order; fair 1.918 vs best 1.887.</t>
+      <c r="I10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="6" t="n"/>
+      <c r="K10" s="6" t="n"/>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>Saturday sources split (CIN 2.05 vs 2.20); best price sits near fair. Premise risk: sources conflict on whether Skenes starts Saturday or pitched Friday - if Skenes is gone, the CIN side strengthens.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>PIT @ CIN</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Pirates ML</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>order_open</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>1.874</v>
+      </c>
+      <c r="F11" s="3" t="n"/>
+      <c r="G11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="6" t="n"/>
+      <c r="K11" s="6" t="n"/>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>Runner-up order; fair 1.828 vs best 1.80.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>NYY @ CHC</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Market refused (conflict rule, day 2)</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>refusal</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="n"/>
+      <c r="F12" s="3" t="n"/>
+      <c r="G12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="6" t="n"/>
+      <c r="K12" s="6" t="n"/>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>conflict</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>Books: Cubs 1.62; Polymarket: Yankees favored. Same signature the close resolved toward books yesterday (-11.67% pseudo-hold). Saturday pitchers also unresolved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>WSH @ ATL</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Market refused (no anchor &gt;= 0.5)</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>refusal</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="n"/>
+      <c r="F13" s="3" t="n"/>
+      <c r="G13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="6" t="n"/>
+      <c r="K13" s="6" t="n"/>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>Only Polymarket quotes both sides; after its ledger-evidenced demotion to 0.45 it cannot anchor a fair line.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>Blue cells = ledger data (regenerated by sharpods-tracker; edit data/track_record.json, not this sheet). Dashboard recomputes from these rows automatically. To grade a bet you placed yourself: set Type=ticket, Result=won or lost, and fill Stake $ and P&amp;L $ — the Dashboard picks it up. For an order that never filled, set Result=no fill.</t>
         </is>
@@ -1052,7 +1264,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1387,14 +1599,14 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>mlb-2026-07-30-nyy-cws</t>
+          <t>mlb-2026-07-30-mia-nym</t>
         </is>
       </c>
       <c r="C9" s="8" t="n">
-        <v>0.4317</v>
+        <v>0.5522</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>0.5115</v>
+        <v>0.5454</v>
       </c>
       <c r="E9" s="9">
         <f>ABS(C9-D9)*100</f>
@@ -1413,7 +1625,159 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
+          <t>clean</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>mlb-2026-07-30-wsh-atl</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="n">
+        <v>0.5255</v>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>0.5665</v>
+      </c>
+      <c r="E10" s="9">
+        <f>ABS(C10-D10)*100</f>
+        <v/>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="10">
+        <f>(C10-F10)^2</f>
+        <v/>
+      </c>
+      <c r="H10" s="10">
+        <f>(D10-F10)^2</f>
+        <v/>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>stale quote</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>mlb-2026-07-30-bos-ath</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="n">
+        <v>0.4117</v>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>0.3733</v>
+      </c>
+      <c r="E11" s="9">
+        <f>ABS(C11-D11)*100</f>
+        <v/>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="10">
+        <f>(C11-F11)^2</f>
+        <v/>
+      </c>
+      <c r="H11" s="10">
+        <f>(D11-F11)^2</f>
+        <v/>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>low-conf close</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>mlb-2026-07-30-nyy-cws</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="n">
+        <v>0.4317</v>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>0.5115</v>
+      </c>
+      <c r="E12" s="9">
+        <f>ABS(C12-D12)*100</f>
+        <v/>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="10">
+        <f>(C12-F12)^2</f>
+        <v/>
+      </c>
+      <c r="H12" s="10">
+        <f>(D12-F12)^2</f>
+        <v/>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
           <t>date trap</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>mlb-2026-07-30-sea-lad</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="n">
+        <v>0.5883</v>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>0.5934</v>
+      </c>
+      <c r="E13" s="9">
+        <f>ABS(C13-D13)*100</f>
+        <v/>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="10">
+        <f>(C13-F13)^2</f>
+        <v/>
+      </c>
+      <c r="H13" s="10">
+        <f>(D13-F13)^2</f>
+        <v/>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>clean</t>
         </is>
       </c>
     </row>
@@ -1428,7 +1792,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B34"/>
+  <dimension ref="A1:B37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1700,19 +2064,40 @@
     <row r="31">
       <c r="A31" s="21" t="inlineStr">
         <is>
-          <t>[DIDN'T] CHC @ STL: Cashed on variance: close (CHC +100/STL -120, sharp money on STL) says the edge was not there. Fair missed the no-vig close by 3.7pts on a source-conflict market -&gt; conflict-refusal rule shipped.</t>
+          <t>[WORKED] NYY @ CHC: Close CHC -140 landed on the sportsbook consensus; Polymarket 52c was the stale outlier (NYY won 2-0 as a +130 dog - vs the close that bet was -7% EV luck). Refusal correct.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="21" t="inlineStr">
         <is>
-          <t>[DIDN'T] Calibration: flagged-source fair lines (conflict / date trap / low-confidence close) missed the no-vig close by 5.56 pts on average vs 0.76 pts for clean sources — source hygiene IS calibration.</t>
+          <t>[WORKED] PHI @ BAL: PHI never traded above 2.06 (target 2.10). Close no-vig PHI 0.467: even at target the bet was -2% vs close - not filling saved money. SportsGrid model lean (PHI 54%) was the wrong side per the close.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="21" t="inlineStr">
+        <is>
+          <t>[WORKED] PIT @ CIN: PIT -120 to -136 all day, never near the 1.966 target. Close no-vig PIT 0.564: a 1.966 fill would have been ~+11% EV vs close - right side, market never paid the price.</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="22" t="inlineStr">
+      <c r="A34" s="21" t="inlineStr">
+        <is>
+          <t>[DIDN'T] CHC @ STL: Cashed on variance: close (CHC +100/STL -120, sharp money on STL) says the edge was not there. Fair missed the no-vig close by 3.7pts on a source-conflict market -&gt; conflict-refusal rule shipped.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="21" t="inlineStr">
+        <is>
+          <t>[DIDN'T] Calibration: flagged-source fair lines (conflict / date trap / low-confidence close) missed the no-vig close by 4.93 pts on average vs 0.72 pts for clean sources — source hygiene IS calibration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="22" t="inlineStr">
         <is>
           <t>Source: data/track_record.json (SharpOds ledger); regenerated by `sharpods-tracker`. Assumption: closing lines are best-available day-of published numbers, not exchange-verified closing ticks.</t>
         </is>

</xml_diff>

<commit_message>
Ship Aug 1 all-sports card; tracker shows the daily best bet only
Final multi-sport run (11 MLB + 3 UFC + CFL spread + 2 WNBA = 20 markets,
3 refusals): best bet Reds ML, order at >= 2.242. Ledger decisions carry
headline flags; the tracker filters to one card per day matching the
user's stated behavior of betting only the slip's best bet.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Epz958ydWx4TMSQvnKeiSm
</commit_message>
<xml_diff>
--- a/data/tracker.xlsx
+++ b/data/tracker.xlsx
@@ -1056,7 +1056,7 @@
         </is>
       </c>
       <c r="E10" s="3" t="n">
-        <v>2.262</v>
+        <v>2.242</v>
       </c>
       <c r="F10" s="3" t="n"/>
       <c r="G10" s="4" t="n">
@@ -1084,7 +1084,7 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>Saturday sources split (CIN 2.05 vs 2.20); best price sits near fair. Premise risk: sources conflict on whether Skenes starts Saturday or pitched Friday - if Skenes is gone, the CIN side strengthens.</t>
+          <t>Best bet of the multi-sport card. Saturday sources split on CIN (2.05 vs 2.20); best price near fair 2.188 and the Stats Insider model (CIN 48%) nudges it up. Premise: Ashcraft (PIT) vs LHP Abbott (CIN), 6:40 PM ET - Skenes pitched Friday.</t>
         </is>
       </c>
     </row>
@@ -1110,7 +1110,7 @@
         </is>
       </c>
       <c r="E11" s="3" t="n">
-        <v>1.874</v>
+        <v>1.888</v>
       </c>
       <c r="F11" s="3" t="n"/>
       <c r="G11" s="4" t="n">
@@ -1138,7 +1138,7 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>Runner-up order; fair 1.828 vs best 1.80.</t>
+          <t>Runner-up order; fair 1.842 vs best 1.80.</t>
         </is>
       </c>
     </row>
@@ -1190,7 +1190,7 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>Books: Cubs 1.62; Polymarket: Yankees favored. Same signature the close resolved toward books yesterday (-11.67% pseudo-hold). Saturday pitchers also unresolved.</t>
+          <t>Books: Cubs 1.62; Polymarket: Yankees favored (-11.67% pseudo-hold) - day-2 conflict. Saturday pitchers unresolved (Warren vs Imanaga was Friday's game, which NYY won 2-0). Refusal graded at Saturday's close.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Complete Aug 1 all-sports card: 49 markets, soccer live, best bet found
Fix round closes every identified gap: 8 soccer three-way markets (5 MLS
+ 2 Liga MX + models), MLB run lines/totals for 5 games plus the two
missing boards, full 14-bout UFC card, CFL two-sided, in-house log5 on
verified records in 8 blends. Two bugs fixed (Wong teasers gated to
football; WNBA Liberty-at-Phoenix venue reversal) and two data traps
caught (Friday Mariners line, garbled Galaxy-Dallas quote). Final run:
one bet clears the bar - Timbers ML at 2.273 on the prediction market vs
the bet365-anchored fair 2.175 (+4.51% EV, robust under either price) -
with Orioles >= 2.225 and Reds >= 2.231 as backup orders.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Epz958ydWx4TMSQvnKeiSm
</commit_message>
<xml_diff>
--- a/data/tracker.xlsx
+++ b/data/tracker.xlsx
@@ -511,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1056,7 +1056,7 @@
         </is>
       </c>
       <c r="E10" s="3" t="n">
-        <v>2.242</v>
+        <v>2.231</v>
       </c>
       <c r="F10" s="3" t="n"/>
       <c r="G10" s="4" t="n">
@@ -1084,7 +1084,7 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>Best bet of the multi-sport card. Saturday sources split on CIN (2.05 vs 2.20); best price near fair 2.188 and the Stats Insider model (CIN 48%) nudges it up. Premise: Ashcraft (PIT) vs LHP Abbott (CIN), 6:40 PM ET - Skenes pitched Friday.</t>
+          <t>Runner-up on the full card (was headline on the draft). Fair 2.176 with in-house log5 (CIN 51.2% by records) ensembled with Stats Insider (48%). Ashcraft vs Abbott.</t>
         </is>
       </c>
     </row>
@@ -1118,7 +1118,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>superseded</t>
         </is>
       </c>
       <c r="I11" s="5" t="n">
@@ -1138,7 +1138,7 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>Runner-up order; fair 1.842 vs best 1.80.</t>
+          <t>Superseded by the full-card re-rank (PIT side fell out of the top orders).</t>
         </is>
       </c>
     </row>
@@ -1246,8 +1246,116 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>PHI @ BAL</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Orioles ML</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>order_open</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>2.225</v>
+      </c>
+      <c r="F14" s="3" t="n"/>
+      <c r="G14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="6" t="n"/>
+      <c r="K14" s="6" t="n"/>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>Best bet of the full all-sports card. Market prices PHI -130 despite PHI 2-8 last ten and a hot Baltimore (ESPN Analytics 55.5% BAL). Fair 2.171; order fires at 2.225+. Sanchez vs Baz, 7:05 PM ET Camden Yards. Caveat: single-book price (FanDuel via Covers), BAL record stale in our in-house layer - model prob is ESPN-only.</t>
+        </is>
+      </c>
+    </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>SEA @ POR (MLS)</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Timbers ML</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>order_open</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>2.273</v>
+      </c>
+      <c r="F15" s="3" t="n"/>
+      <c r="G15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="6" t="n"/>
+      <c r="K15" s="6" t="n"/>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>BEST BET - the only bar-clearing play on the 49-market card. Prediction market pays 2.273 (44c) on a side bet365 prices 2.05; fair 2.175 -&gt; +4.51% EV, robust under either price being true. Fill condition: Portland at 44c or better; if the ask has moved above 44c, the edge shrinks - engine minimum price 2.23 (45c). Providence Park, ~10:30 PM ET.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>Blue cells = ledger data (regenerated by sharpods-tracker; edit data/track_record.json, not this sheet). Dashboard recomputes from these rows automatically. To grade a bet you placed yourself: set Type=ticket, Result=won or lost, and fill Stake $ and P&amp;L $ — the Dashboard picks it up. For an order that never filled, set Result=no fill.</t>
         </is>

</xml_diff>

<commit_message>
Regrade Timbers headline as no-fill per user execution report
The prediction-market ask moved above the 45c stand-down line before bet
time, so per the slip's fill rule no bet was placed - the user correctly
stood down. Decision regraded from won ticket to unfilled order (paper
CLV of the 2.273 snapshot kept in the note); tickets revert to 1-0.
Lessons updated: prediction-market discounts are real edge with a
narrow execution window, and the user's report is the only fill oracle
(pages 403 post-hoc). Grade orders on fills, never on hindsight.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Epz958ydWx4TMSQvnKeiSm
</commit_message>
<xml_diff>
--- a/data/tracker.xlsx
+++ b/data/tracker.xlsx
@@ -1318,32 +1318,26 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>ticket</t>
+          <t>order_unfilled</t>
         </is>
       </c>
       <c r="E15" s="3" t="n">
-        <v>2.273</v>
-      </c>
-      <c r="F15" s="3" t="n">
-        <v>2.273</v>
-      </c>
+        <v>2.23</v>
+      </c>
+      <c r="F15" s="3" t="n"/>
       <c r="G15" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>won</t>
+          <t>no fill</t>
         </is>
       </c>
       <c r="I15" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="J15" s="6" t="n">
-        <v>0.1088</v>
-      </c>
-      <c r="K15" s="6" t="n">
-        <v>0.0451</v>
-      </c>
+      <c r="J15" s="6" t="n"/>
+      <c r="K15" s="6" t="n"/>
       <c r="L15" s="2" t="inlineStr">
         <is>
           <t>clean</t>
@@ -1356,7 +1350,7 @@
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>WON - Portland 2-1 Seattle. Graded at the pre-registered listed price 2.273 (prediction-market 44c; post-hoc fill verification impossible, page 403s). bet365 close 2.05/3.80/3.00: raw CLV +10.9%, no-vig CLV +4.5% - first positive-CLV ticket. User stake unconfirmed (no ticket screenshot); tracker computes P&amp;L at your unit stake.</t>
+          <t>NO BET - user report (the only fill oracle; pages 403 post-hoc): the prediction-market ask had moved above the 45c stand-down line (engine minimum 2.23) by bet time, so per the slip's own fill rule the order did not fire. Paper grade of the 2.273 listed snapshot: Portland won 2-1 and the number beat the bet365 close 2.05/3.80/3.00 by +10.9% raw / +4.5% no-vig - the edge was real at the snapshot, and it decayed before execution. Standing down was correct: at the moved ask the +2.5% EV bar was no longer met.</t>
         </is>
       </c>
     </row>
@@ -2859,7 +2853,7 @@
     <row r="38">
       <c r="A38" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] SEA @ POR (MLS): WON - Portland 2-1 Seattle. Graded at the pre-registered listed price 2.273 (prediction-market 44c; post-hoc fill verification impossible, page 403s). bet365 close 2.05/3.80/3.00: raw CLV +10.9%, no-vig CLV +4.5% - first positive-CLV ticket. User stake unconfirmed (no ticket screenshot); tracker computes P&amp;L at your unit stake.</t>
+          <t>[WORKED] SEA @ POR (MLS): NO BET - user report (the only fill oracle; pages 403 post-hoc): the prediction-market ask had moved above the 45c stand-down line (engine minimum 2.23) by bet time, so per the slip's own fill rule the order did not fire. Paper grade of the 2.273 listed snapshot: Portland won 2-1 and the number beat the bet365 close 2.05/3.80/3.00 by +10.9% raw / +4.5% no-vig - the edge was real at the snapshot, and it decayed before execution. Standing down was correct: at the moved ask the +2.5% EV bar was no longer met.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Void the Aug 2 orders (card shipped after first pitch) and add staleness gate
User caught the miss: the headline order (WSH@ATL, 1:35 PM ET) shipped
hours after the game started. Root cause: the container clock said
Sunday evening, search snippets showed no Sunday finals, and the
optimistic reading won - but a lagging search index cannot prove
pre-game. All three orders voided in the ledger (no fills, no hindsight
grading); the day stands as a full pass either way (best EV was -0.04%).

Protocol hardened in CLAUDE.md: 'now' for staleness decisions is the
most pessimistic of clock vs evidence, and a new ship-time gate blocks
any pick whose start time is not 2+ hours past pessimistic-now - if
nothing qualifies, ship the next day's card instead.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Epz958ydWx4TMSQvnKeiSm
</commit_message>
<xml_diff>
--- a/data/tracker.xlsx
+++ b/data/tracker.xlsx
@@ -1372,7 +1372,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>order_open</t>
+          <t>order_void</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -1384,7 +1384,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>no fill</t>
         </is>
       </c>
       <c r="I16" s="5" t="n">
@@ -1399,12 +1399,12 @@
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>miss</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>BEST ORDER on a pass card - nothing is bettable at listed prices today. Fair 1.821 (market 0.5325 blended with in-house log5 0.6408 at 85/15); order fires only at 1.866+ (+2.5% EV bar). CAVEAT, stated plainly: 80% of sharp ML handle is on WSH fading ATL's rookie spot-starter JR Ritchie - our records-only log5 cannot see pitching. If the line moves toward the order, it is moving against the sharps. Bet the number or nothing.</t>
+          <t>VOID - PROCESS MISS (user report): the card shipped hours after this game's 1:35 PM ET first pitch. The container clock read Sunday evening; I overrode it because search snippets showed no Sunday finals - but a lagging search index is not pre-game proof. Order was never actionable; no bet placed, none should be. Original order terms preserved above for the record; outcome deliberately NOT graded (no hindsight grading of a void order).</t>
         </is>
       </c>
     </row>
@@ -1426,7 +1426,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>order_open</t>
+          <t>order_void</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
@@ -1438,7 +1438,7 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>no fill</t>
         </is>
       </c>
       <c r="I17" s="5" t="n">
@@ -1453,12 +1453,12 @@
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>miss</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>Fair 1.626 off the Caesars 1.625 board (DK is shaded to 1.541); in-house log5 agrees with the market (LAD 62.5%). BOS won Fri+Sat - if steam keeps pushing BOS, LAD 1.666+ becomes available. Bennett vs Sheehan.</t>
+          <t>VOID - cancelled at 7:03 PM ET with first pitch 7:20 PM ET: no time to re-verify the line, and every price on the card is a morning-stale snapshot. An unsupervisable order is not an order.</t>
         </is>
       </c>
     </row>
@@ -1480,7 +1480,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>order_open</t>
+          <t>order_void</t>
         </is>
       </c>
       <c r="E18" s="3" t="n">
@@ -1492,7 +1492,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>no fill</t>
         </is>
       </c>
       <c r="I18" s="5" t="n">
@@ -1507,12 +1507,12 @@
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>miss</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>Strongest situational thesis on the card: Alcantara vs an emergency spot starter (Robert Stock), SportsGrid 56% MIA, in-house log5 55.5% MIA. Fair 1.878; needs +108 -&gt; +115ish to fire.</t>
+          <t>VOID - shipped after the 1:40 PM ET first pitch (same process miss as the headline order). No bet placed, none should be.</t>
         </is>
       </c>
     </row>
@@ -2532,7 +2532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B42"/>
+  <dimension ref="A1:B45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2867,12 +2867,33 @@
     <row r="40">
       <c r="A40" s="21" t="inlineStr">
         <is>
+          <t>[DIDN'T] WSH @ ATL: VOID - PROCESS MISS (user report): the card shipped hours after this game's 1:35 PM ET first pitch. The container clock read Sunday evening; I overrode it because search snippets showed no Sunday finals - but a lagging search index is not pre-game proof. Order was never actionable; no bet placed, none should be. Original order terms preserved above for the record; outcome deliberately NOT graded (no hindsight grading of a void order).</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="21" t="inlineStr">
+        <is>
+          <t>[DIDN'T] BOS @ LAD (Sunday Night Baseball): VOID - cancelled at 7:03 PM ET with first pitch 7:20 PM ET: no time to re-verify the line, and every price on the card is a morning-stale snapshot. An unsupervisable order is not an order.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="21" t="inlineStr">
+        <is>
+          <t>[DIDN'T] MIA @ NYM: VOID - shipped after the 1:40 PM ET first pitch (same process miss as the headline order). No bet placed, none should be.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="21" t="inlineStr">
+        <is>
           <t>[DIDN'T] Calibration: flagged-source fair lines (conflict / date trap / low-confidence close) missed the no-vig close by 4.93 pts on average vs 2.27 pts for clean sources — source hygiene IS calibration.</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="22" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="22" t="inlineStr">
         <is>
           <t>Source: data/track_record.json (SharpOds ledger); regenerated by `sharpods-tracker`. Assumption: closing lines are best-available day-of published numbers, not exchange-verified closing ticks.</t>
         </is>

</xml_diff>

<commit_message>
Ship Monday Aug 10 card: 4th straight pass, Skubal game refused on conflict
Compile the Monday night slate (13 events / 15 markets: 9 MLB boards all
7 PM ET+, both WTA Toronto QFs, Tempo@Dream ML, Union-C.Cordoba trio)
with in-house log5 restricted to Aug-4+-verified records and the CIN
conflict resolved. First mid-card ship-time-gate exclusion: the ATP
Jodar-Fils QF's pessimistic start (12:35 PM ET) sits inside the runway.
Engine verdict: PASS - top orders Braves ML >= 1.684 (headline, EV now
-0.34%), Swiatek >= 1.403, D-backs >= 1.624. REFUSED: KC@LAD (Skubal
home debut) - book 1.625 vs Polymarket 1.351 = -12.95% cross-source
hold, the widest conflict recorded; rule applied a 5th time. Excluded
by name: MIL@SD Frankenstein pair, CHI@SEA favorite contradiction, two
aggregate soccer trios, Tempo@Dream spread/total dispersion.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Epz958ydWx4TMSQvnKeiSm
</commit_message>
<xml_diff>
--- a/data/tracker.xlsx
+++ b/data/tracker.xlsx
@@ -511,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N29"/>
+  <dimension ref="A1:N33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1806,7 +1806,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>order_open</t>
+          <t>order_unfilled</t>
         </is>
       </c>
       <c r="E24" s="3" t="n">
@@ -1818,7 +1818,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>no fill</t>
         </is>
       </c>
       <c r="I24" s="5" t="n">
@@ -1833,12 +1833,12 @@
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>worked</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>HEADLINE ORDER on a market-only card. Fair 1.638 (pure power-devig of the Covers single-book board CIN -171/ATH +141; no model - CIN's published records conflict arithmetically with our verified baseline, so the in-house layer sits out rather than eat bad input). Fires at 1.679+ only. Caveats: Aug-6 pitchers unannounced at ship time; single-book anchor; verify the start time before acting - the gate clears even at the earliest plausible start, but a fill needs a live re-check of pitchers and price.</t>
+          <t>NOT FILLED: CIN drifted our way (-171 open -&gt; -158 at first pitch) but never reached the -147 (1.679) bar; best documented 1.633. CIN won 6-5, and a 1.679 fill would have carried +2.8% raw CLV vs the close - right side, right price demand, market never paid it. Reverse line movement toward the road dog noted pregame; the bar held anyway.</t>
         </is>
       </c>
     </row>
@@ -1860,7 +1860,7 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>order_open</t>
+          <t>order_unfilled</t>
         </is>
       </c>
       <c r="E25" s="3" t="n">
@@ -1872,7 +1872,7 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>no fill</t>
         </is>
       </c>
       <c r="I25" s="5" t="n">
@@ -1887,12 +1887,12 @@
       </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>worked</t>
         </is>
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>Engine's top order by EV, deliberately NOT the headline: on a 1.10 favorite, a 4-cent 'fill' is usually cross-book variance, not a market move - the Aug-3 Liberty grade showed resting-trigger fills on drifting lines carry negative CLV. This order requires a re-verified live quote at 1.141+, not a resting fill.</t>
+          <t>NOT FILLED: Braga sat 1.10-1.11 everywhere pre-match; the 1.141 re-verified quote never existed. Braga won 1-0. The demotion logic validated exactly: on extreme favorites the only 'fills' available are cross-book noise, and even that noise stayed under 4 cents.</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>order_open</t>
+          <t>order_unfilled</t>
         </is>
       </c>
       <c r="E26" s="3" t="n">
@@ -1926,7 +1926,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>no fill</t>
         </is>
       </c>
       <c r="I26" s="5" t="n">
@@ -1941,12 +1941,12 @@
       </c>
       <c r="M26" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>worked</t>
         </is>
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>First football order of the season, strictly a backup. Fair 1.834 off the DK board; juice already flipped toward the ARI side (dog money). PRESEASON: starters sit, Carson Beck starts for ARI, variance extreme - star sizing only if it somehow fills.</t>
+          <t>NOT FILLED by one cent of juice: ARI +1.5 reached ~-115 game-day vs the -114 bar - and then LOST (CAR won by exactly 3 on the final play). The near-miss dodged a loser; fill discipline is net positive on the card (two would-have-won fills never reached target, the one would-have-lost fill missed by a cent).</t>
         </is>
       </c>
     </row>
@@ -1978,7 +1978,7 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>validated</t>
         </is>
       </c>
       <c r="I27" s="5" t="n">
@@ -1993,17 +1993,231 @@
       </c>
       <c r="M27" s="2" t="inlineStr">
         <is>
+          <t>worked</t>
+        </is>
+      </c>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>Suppression validated on process with an ironic outcome: the suppressed leg (ARI +1.5 -&gt; +7.5) would have back-doored a win (lost by 3), but the game produced 63 points against a 34.5 total - preseason margins have NO key-number structure, which is precisely why the leg had no business existing. Note-only; engine gating change still deferred (Walters rule).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>NYM @ ATL (7:15 PM ET Mon)</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Braves ML</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>order_open</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>1.684</v>
+      </c>
+      <c r="F28" s="3" t="n"/>
+      <c r="G28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
           <t>pending</t>
         </is>
       </c>
-      <c r="N27" s="2" t="inlineStr">
-        <is>
-          <t>The teaser machinery is correctly football-gated, but preseason football lacks the key-number margin distribution Wong teasers exploit (starters sit; 3s and 7s aren't privileged). Leg suppressed from the slip by hand; a preseason/regular-season gate in the engine is deferred until a graded miss justifies it (Walters rule). This flag is that paper trail.</t>
+      <c r="I28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" s="6" t="n"/>
+      <c r="K28" s="6" t="n"/>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>HEADLINE ORDER. Fair 1.643 (market 0.590 blended 85/15 with in-house log5 0.708 - ATL 69-45 vs NYM 49-66, model and market agree on direction). Fires at 1.684+ (needs a 4-5 cent drift from -157). Scott vs Elder (3.00 home ERA). If it fills: $92 at quarter-Kelly (0.92%), returns $155. Re-verify the price live - order, not a bet.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="7" t="inlineStr">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Shnaider vs Swiatek, WTA Toronto QF (7:00 PM ET Mon)</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Swiatek ML</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>order_open</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="n">
+        <v>1.403</v>
+      </c>
+      <c r="F29" s="3" t="n"/>
+      <c r="G29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="I29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" s="6" t="n"/>
+      <c r="K29" s="6" t="n"/>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>Fair 1.369 (market 0.729 blended with Dimers 74%). Book range already spans -285/-300; a 1.403 (+/-248) print at a real book fires it. Short-price order - small sizing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>COL @ AZ (Chase Field, evening - exact time TBC)</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Diamondbacks ML</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>order_open</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="n">
+        <v>1.624</v>
+      </c>
+      <c r="F30" s="3" t="n"/>
+      <c r="G30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="I30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" s="6" t="n"/>
+      <c r="K30" s="6" t="n"/>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>Fair 1.584 (market 0.623 + in-house 0.676 - AZ 63-56 vs COL 45-71). Verify the start time before acting; even the earliest plausible window clears the gate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>KC @ LAD (10:10 PM ET Mon - Skubal home debut)</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Moneyline refused (conflict rule)</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>refusal</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="n"/>
+      <c r="F31" s="3" t="n"/>
+      <c r="G31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="I31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" s="6" t="n"/>
+      <c r="K31" s="6" t="n"/>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>conflict</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>Book prices LAD 1.625 (-160); Polymarket pays 1.351 (74c) on the same side - cross-source hold -12.95%, the widest conflict we've recorded. Degraded anchor + negative hold = unpriceable, never an arb (rule now applied a 5th time; 4-for-4 validated so far). The hype game is exactly where quote quality dies. Graded at Monday's close.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
         <is>
           <t>Blue cells = ledger data (regenerated by sharpods-tracker; edit data/track_record.json, not this sheet). Dashboard recomputes from these rows automatically. To grade a bet you placed yourself: set Type=ticket, Result=won or lost, and fill Stake $ and P&amp;L $ — the Dashboard picks it up. For an order that never filled, set Result=no fill.</t>
         </is>
@@ -2020,7 +2234,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:I52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3905,6 +4119,120 @@
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>mlb-2026-08-06-ath-cin</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="n">
+        <v>0.6104000000000001</v>
+      </c>
+      <c r="D50" s="8" t="n">
+        <v>0.6038</v>
+      </c>
+      <c r="E50" s="9">
+        <f>ABS(C50-D50)*100</f>
+        <v/>
+      </c>
+      <c r="F50" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G50" s="10">
+        <f>(C50-F50)^2</f>
+        <v/>
+      </c>
+      <c r="H50" s="10">
+        <f>(D50-F50)^2</f>
+        <v/>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>nfl-2026-08-06-ari-car</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="n">
+        <v>0.5112</v>
+      </c>
+      <c r="D51" s="8" t="n">
+        <v>0.5302</v>
+      </c>
+      <c r="E51" s="9">
+        <f>ABS(C51-D51)*100</f>
+        <v/>
+      </c>
+      <c r="F51" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G51" s="10">
+        <f>(C51-F51)^2</f>
+        <v/>
+      </c>
+      <c r="H51" s="10">
+        <f>(D51-F51)^2</f>
+        <v/>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>uecl-2026-08-06-din-bra</t>
+        </is>
+      </c>
+      <c r="C52" s="8" t="n">
+        <v>0.898</v>
+      </c>
+      <c r="D52" s="8" t="n">
+        <v>0.898</v>
+      </c>
+      <c r="E52" s="9">
+        <f>ABS(C52-D52)*100</f>
+        <v/>
+      </c>
+      <c r="F52" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G52" s="10">
+        <f>(C52-F52)^2</f>
+        <v/>
+      </c>
+      <c r="H52" s="10">
+        <f>(D52-F52)^2</f>
+        <v/>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3916,7 +4244,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B49"/>
+  <dimension ref="A1:B53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -4272,40 +4600,68 @@
     <row r="43">
       <c r="A43" s="21" t="inlineStr">
         <is>
-          <t>[DIDN'T] CHC @ STL: Cashed on variance: close (CHC +100/STL -120, sharp money on STL) says the edge was not there. Fair missed the no-vig close by 3.7pts on a source-conflict market -&gt; conflict-refusal rule shipped.</t>
+          <t>[WORKED] ATH @ CIN (start time unverified; typical 12:35 PM ET getaway): NOT FILLED: CIN drifted our way (-171 open -&gt; -158 at first pitch) but never reached the -147 (1.679) bar; best documented 1.633. CIN won 6-5, and a 1.679 fill would have carried +2.8% raw CLV vs the close - right side, right price demand, market never paid it. Reverse line movement toward the road dog noted pregame; the bar held anyway.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="21" t="inlineStr">
         <is>
-          <t>[DIDN'T] WSH @ ATL: VOID - PROCESS MISS (user report): the card shipped hours after this game's 1:35 PM ET first pitch. The container clock read Sunday evening; I overrode it because search snippets showed no Sunday finals - but a lagging search index is not pre-game proof. Order was never actionable; no bet placed, none should be. Original order terms preserved above for the record; outcome deliberately NOT graded (no hindsight grading of a void order).</t>
+          <t>[WORKED] Dinamo Minsk @ Braga (UECL Q3 leg 1; kickoff ~3:00-3:45 PM ET assumed): NOT FILLED: Braga sat 1.10-1.11 everywhere pre-match; the 1.141 re-verified quote never existed. Braga won 1-0. The demotion logic validated exactly: on extreme favorites the only 'fills' available are cross-book noise, and even that noise stayed under 4 cents.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="21" t="inlineStr">
         <is>
-          <t>[DIDN'T] BOS @ LAD (Sunday Night Baseball): VOID - cancelled at 7:03 PM ET with first pitch 7:20 PM ET: no time to re-verify the line, and every price on the card is a morning-stale snapshot. An unsupervisable order is not an order.</t>
+          <t>[WORKED] ARI @ CAR, Hall of Fame Game (8:00 PM ET Thu, Canton - neutral site): NOT FILLED by one cent of juice: ARI +1.5 reached ~-115 game-day vs the -114 bar - and then LOST (CAR won by exactly 3 on the final play). The near-miss dodged a loser; fill discipline is net positive on the card (two would-have-won fills never reached target, the one would-have-lost fill missed by a cent).</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="21" t="inlineStr">
         <is>
-          <t>[DIDN'T] MIA @ NYM: VOID - shipped after the 1:40 PM ET first pitch (same process miss as the headline order). No bet placed, none should be.</t>
+          <t>[WORKED] ARI @ CAR (HOF Game): Suppression validated on process with an ironic outcome: the suppressed leg (ARI +1.5 -&gt; +7.5) would have back-doored a win (lost by 3), but the game produced 63 points against a 34.5 total - preseason margins have NO key-number structure, which is precisely why the leg had no business existing. Note-only; engine gating change still deferred (Walters rule).</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="21" t="inlineStr">
         <is>
-          <t>[DIDN'T] Calibration: flagged-source fair lines (conflict / date trap / low-confidence close) missed the no-vig close by 4.93 pts on average vs 1.66 pts for clean sources — source hygiene IS calibration.</t>
+          <t>[DIDN'T] CHC @ STL: Cashed on variance: close (CHC +100/STL -120, sharp money on STL) says the edge was not there. Fair missed the no-vig close by 3.7pts on a source-conflict market -&gt; conflict-refusal rule shipped.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="21" t="inlineStr">
+        <is>
+          <t>[DIDN'T] WSH @ ATL: VOID - PROCESS MISS (user report): the card shipped hours after this game's 1:35 PM ET first pitch. The container clock read Sunday evening; I overrode it because search snippets showed no Sunday finals - but a lagging search index is not pre-game proof. Order was never actionable; no bet placed, none should be. Original order terms preserved above for the record; outcome deliberately NOT graded (no hindsight grading of a void order).</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="22" t="inlineStr">
+      <c r="A49" s="21" t="inlineStr">
+        <is>
+          <t>[DIDN'T] BOS @ LAD (Sunday Night Baseball): VOID - cancelled at 7:03 PM ET with first pitch 7:20 PM ET: no time to re-verify the line, and every price on the card is a morning-stale snapshot. An unsupervisable order is not an order.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="21" t="inlineStr">
+        <is>
+          <t>[DIDN'T] MIA @ NYM: VOID - shipped after the 1:40 PM ET first pitch (same process miss as the headline order). No bet placed, none should be.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="21" t="inlineStr">
+        <is>
+          <t>[DIDN'T] Calibration: flagged-source fair lines (conflict / date trap / low-confidence close) missed the no-vig close by 4.93 pts on average vs 1.61 pts for clean sources — source hygiene IS calibration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="22" t="inlineStr">
         <is>
           <t>Source: data/track_record.json (SharpOds ledger); regenerated by `sharpods-tracker`. Assumption: closing lines are best-available day-of published numbers, not exchange-verified closing ticks.</t>
         </is>

</xml_diff>

<commit_message>
Update Sep 9 slip and tracker: order stood down
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Epz958ydWx4TMSQvnKeiSm
</commit_message>
<xml_diff>
--- a/data/tracker.xlsx
+++ b/data/tracker.xlsx
@@ -4584,7 +4584,7 @@
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>order_open</t>
+          <t>order_cancelled</t>
         </is>
       </c>
       <c r="E75" s="3" t="n">
@@ -4596,7 +4596,7 @@
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>cancelled - premise changed</t>
         </is>
       </c>
       <c r="I75" s="5" t="n">
@@ -4611,12 +4611,12 @@
       </c>
       <c r="M75" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>worked</t>
         </is>
       </c>
       <c r="N75" s="2" t="inlineStr">
         <is>
-          <t>HEADLINE ORDER - dispersion tier (+1.0% bar; Kalshi at 0.45 sharpness sits below the 0.50 fair-line floor, so it is a shop venue, never a fair source). Fires at 37c or better (2.7027, +170). Blended fair 2.675 (37.38%); the model ensemble alone says 39.33%, so a 37c fill is +1.03% on the blend and +6.30% on the model. Best live prices: BetRivers +160 (a fair source, so it carries the +1.5% model-tier bar = 2.715 and misses), Kalshi 39c = 2.5641. TWO BINDING CLAUSES. (1) DRIFT-CANCEL WITH A NAMED TRIGGER: TreVeyon Henderson (NE RB) has not practiced since Aug 24 and his final designation was still outstanding at compile. If New England reaches 37c ON A HENDERSON-OUT HEADLINE, that is a drift, not a fill - the premise our fair was built on changed, the true probability moved down with the price, and we stand down and re-price. A 37c print on ordinary two-way flow with no news is a legitimate standing-above fill. Both graded drift-fills (Liberty Aug-3, Braves Aug-10) arrived exactly this way and both carried negative CLV. (2) BOOK-INTEGRITY FLOOR: the order is void if Kalshi's two legs sum to 100c or less (e.g. NE 36c against SEA 64c). Our own conflict rule refuses a zero/negative synthetic hold on a degraded anchor, and an exchange showing one is showing a stale side, not a gift. Verified at compile: NE 39c + SEA 63c = 102c. PREMISES HELD AT COMPILE: Maye and Darnold both entirely absent from the injury report; NE C Ben Brown OUT. $15 at quarter-Kelly if filled at 37c (returns $41); ~$54 at 36c.</t>
+          <t>HEADLINE ORDER - dispersion tier (+1.0% bar; Kalshi at 0.45 sharpness sits below the 0.50 fair-line floor, so it is a shop venue, never a fair source). Fires at 37c or better (2.7027, +170). Blended fair 2.675 (37.38%); the model ensemble alone says 39.33%, so a 37c fill is +1.03% on the blend and +6.30% on the model. Best live prices: BetRivers +160 (a fair source, so it carries the +1.5% model-tier bar = 2.715 and misses), Kalshi 39c = 2.5641. TWO BINDING CLAUSES. (1) DRIFT-CANCEL WITH A NAMED TRIGGER: TreVeyon Henderson (NE RB) has not practiced since Aug 24 and his final designation was still outstanding at compile. If New England reaches 37c ON A HENDERSON-OUT HEADLINE, that is a drift, not a fill - the premise our fair was built on changed, the true probability moved down with the price, and we stand down and re-price. A 37c print on ordinary two-way flow with no news is a legitimate standing-above fill. Both graded drift-fills (Liberty Aug-3, Braves Aug-10) arrived exactly this way and both carried negative CLV. (2) BOOK-INTEGRITY FLOOR: the order is void if Kalshi's two legs sum to 100c or less (e.g. NE 36c against SEA 64c). Our own conflict rule refuses a zero/negative synthetic hold on a degraded anchor, and an exchange showing one is showing a stale side, not a gift. Verified at compile: NE 39c + SEA 63c = 102c. PREMISES HELD AT COMPILE: Maye and Darnold both entirely absent from the injury report; NE C Ben Brown OUT. $15 at quarter-Kelly if filled at 37c (returns $41); ~$54 at 36c. || CANCELLED Wed 2026-09-09 12:01Z (8:01 AM ET, ~12h pre-kickoff), on the fallback wake. THE NAMED TRIGGER FIRED: TreVeyon Henderson was RULED OUT on New England's final injury report, released Tuesday Sep 8 - the exact condition clause (1) was written against. Market state at cancellation: Kalshi SEA 63c / NE 38c (sum 101c, so the book-integrity floor in clause (2) held). TWO SEPARATE FACTS, and they matter independently. FIRST: the order never filled on its own terms - 38c never reached the 37c trigger, so this is a no-fill regardless of the premise. SECOND: the market moved one cent IN OUR FAVOUR (39c -&gt; 38c, i.e. New England got cheaper), and that is exactly the trap the clause exists to catch - the price improved BECAUSE the true probability fell, not because value appeared. Had the drift carried one more cent to 37c we would have been handed a trigger print on a side whose premise had just deteriorated, which is the shape of both graded drift-fills (Liberty Aug-3, Braves Aug-10) that carried negative CLV. Standing the order down rather than leaving a resting trigger we would not honour. NOT RE-PRICED: a fresh fair would need a new compile, and this is a fallback wake, not a GO. At the compile fair the 38c price is -1.63% on the blend (+3.50% on the model alone), so nothing clears in any case.</t>
         </is>
       </c>
     </row>
@@ -13388,7 +13388,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B98"/>
+  <dimension ref="A1:B99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -14087,40 +14087,47 @@
     <row r="92">
       <c r="A92" s="21" t="inlineStr">
         <is>
-          <t>[DIDN'T] CHC @ STL: Cashed on variance: close (CHC +100/STL -120, sharp money on STL) says the edge was not there. Fair missed the no-vig close by 3.7pts on a source-conflict market -&gt; conflict-refusal rule shipped.</t>
+          <t>[WORKED] Patriots @ Seahawks, NFL Week 1 (8:20 PM ET Wed, Lumen Field): HEADLINE ORDER - dispersion tier (+1.0% bar; Kalshi at 0.45 sharpness sits below the 0.50 fair-line floor, so it is a shop venue, never a fair source). Fires at 37c or better (2.7027, +170). Blended fair 2.675 (37.38%); the model ensemble alone says 39.33%, so a 37c fill is +1.03% on the blend and +6.30% on the model. Best live prices: BetRivers +160 (a fair source, so it carries the +1.5% model-tier bar = 2.715 and misses), Kalshi 39c = 2.5641. TWO BINDING CLAUSES. (1) DRIFT-CANCEL WITH A NAMED TRIGGER: TreVeyon Henderson (NE RB) has not practiced since Aug 24 and his final designation was still outstanding at compile. If New England reaches 37c ON A HENDERSON-OUT HEADLINE, that is a drift, not a fill - the premise our fair was built on changed, the true probability moved down with the price, and we stand down and re-price. A 37c print on ordinary two-way flow with no news is a legitimate standing-above fill. Both graded drift-fills (Liberty Aug-3, Braves Aug-10) arrived exactly this way and both carried negative CLV. (2) BOOK-INTEGRITY FLOOR: the order is void if Kalshi's two legs sum to 100c or less (e.g. NE 36c against SEA 64c). Our own conflict rule refuses a zero/negative synthetic hold on a degraded anchor, and an exchange showing one is showing a stale side, not a gift. Verified at compile: NE 39c + SEA 63c = 102c. PREMISES HELD AT COMPILE: Maye and Darnold both entirely absent from the injury report; NE C Ben Brown OUT. $15 at quarter-Kelly if filled at 37c (returns $41); ~$54 at 36c. || CANCELLED Wed 2026-09-09 12:01Z (8:01 AM ET, ~12h pre-kickoff), on the fallback wake. THE NAMED TRIGGER FIRED: TreVeyon Henderson was RULED OUT on New England's final injury report, released Tuesday Sep 8 - the exact condition clause (1) was written against. Market state at cancellation: Kalshi SEA 63c / NE 38c (sum 101c, so the book-integrity floor in clause (2) held). TWO SEPARATE FACTS, and they matter independently. FIRST: the order never filled on its own terms - 38c never reached the 37c trigger, so this is a no-fill regardless of the premise. SECOND: the market moved one cent IN OUR FAVOUR (39c -&gt; 38c, i.e. New England got cheaper), and that is exactly the trap the clause exists to catch - the price improved BECAUSE the true probability fell, not because value appeared. Had the drift carried one more cent to 37c we would have been handed a trigger print on a side whose premise had just deteriorated, which is the shape of both graded drift-fills (Liberty Aug-3, Braves Aug-10) that carried negative CLV. Standing the order down rather than leaving a resting trigger we would not honour. NOT RE-PRICED: a fresh fair would need a new compile, and this is a fallback wake, not a GO. At the compile fair the 38c price is -1.63% on the blend (+3.50% on the model alone), so nothing clears in any case.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="21" t="inlineStr">
         <is>
-          <t>[DIDN'T] WSH @ ATL: VOID - PROCESS MISS (user report): the card shipped hours after this game's 1:35 PM ET first pitch. The container clock read Sunday evening; I overrode it because search snippets showed no Sunday finals - but a lagging search index is not pre-game proof. Order was never actionable; no bet placed, none should be. Original order terms preserved above for the record; outcome deliberately NOT graded (no hindsight grading of a void order).</t>
+          <t>[DIDN'T] CHC @ STL: Cashed on variance: close (CHC +100/STL -120, sharp money on STL) says the edge was not there. Fair missed the no-vig close by 3.7pts on a source-conflict market -&gt; conflict-refusal rule shipped.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="21" t="inlineStr">
         <is>
-          <t>[DIDN'T] BOS @ LAD (Sunday Night Baseball): VOID - cancelled at 7:03 PM ET with first pitch 7:20 PM ET: no time to re-verify the line, and every price on the card is a morning-stale snapshot. An unsupervisable order is not an order.</t>
+          <t>[DIDN'T] WSH @ ATL: VOID - PROCESS MISS (user report): the card shipped hours after this game's 1:35 PM ET first pitch. The container clock read Sunday evening; I overrode it because search snippets showed no Sunday finals - but a lagging search index is not pre-game proof. Order was never actionable; no bet placed, none should be. Original order terms preserved above for the record; outcome deliberately NOT graded (no hindsight grading of a void order).</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="21" t="inlineStr">
         <is>
-          <t>[DIDN'T] MIA @ NYM: VOID - shipped after the 1:40 PM ET first pitch (same process miss as the headline order). No bet placed, none should be.</t>
+          <t>[DIDN'T] BOS @ LAD (Sunday Night Baseball): VOID - cancelled at 7:03 PM ET with first pitch 7:20 PM ET: no time to re-verify the line, and every price on the card is a morning-stale snapshot. An unsupervisable order is not an order.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="21" t="inlineStr">
         <is>
+          <t>[DIDN'T] MIA @ NYM: VOID - shipped after the 1:40 PM ET first pitch (same process miss as the headline order). No bet placed, none should be.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="21" t="inlineStr">
+        <is>
           <t>[DIDN'T] Calibration: flagged-source fair lines (conflict / date trap / low-confidence close) missed the no-vig close by 4.86 pts on average vs 1.92 pts for clean sources — source hygiene IS calibration.</t>
         </is>
       </c>
     </row>
-    <row r="98">
-      <c r="A98" s="22" t="inlineStr">
+    <row r="99">
+      <c r="A99" s="22" t="inlineStr">
         <is>
           <t>Source: data/track_record.json (SharpOds ledger); regenerated by `sharpods-tracker`. Assumption: closing lines are best-available day-of published numbers, not exchange-verified closing ticks.</t>
         </is>

</xml_diff>

<commit_message>
Regenerate tracker through the Sep 9 settle
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Epz958ydWx4TMSQvnKeiSm
</commit_message>
<xml_diff>
--- a/data/tracker.xlsx
+++ b/data/tracker.xlsx
@@ -4596,14 +4596,16 @@
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>cancelled - premise changed</t>
+          <t>cancelled - never fillable; would have lost</t>
         </is>
       </c>
       <c r="I75" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J75" s="6" t="n"/>
-      <c r="K75" s="6" t="n"/>
+      <c r="K75" s="6" t="n">
+        <v>0.0528</v>
+      </c>
       <c r="L75" s="2" t="inlineStr">
         <is>
           <t>degraded</t>
@@ -4611,12 +4613,12 @@
       </c>
       <c r="M75" s="2" t="inlineStr">
         <is>
-          <t>worked</t>
+          <t>miss</t>
         </is>
       </c>
       <c r="N75" s="2" t="inlineStr">
         <is>
-          <t>HEADLINE ORDER - dispersion tier (+1.0% bar; Kalshi at 0.45 sharpness sits below the 0.50 fair-line floor, so it is a shop venue, never a fair source). Fires at 37c or better (2.7027, +170). Blended fair 2.675 (37.38%); the model ensemble alone says 39.33%, so a 37c fill is +1.03% on the blend and +6.30% on the model. Best live prices: BetRivers +160 (a fair source, so it carries the +1.5% model-tier bar = 2.715 and misses), Kalshi 39c = 2.5641. TWO BINDING CLAUSES. (1) DRIFT-CANCEL WITH A NAMED TRIGGER: TreVeyon Henderson (NE RB) has not practiced since Aug 24 and his final designation was still outstanding at compile. If New England reaches 37c ON A HENDERSON-OUT HEADLINE, that is a drift, not a fill - the premise our fair was built on changed, the true probability moved down with the price, and we stand down and re-price. A 37c print on ordinary two-way flow with no news is a legitimate standing-above fill. Both graded drift-fills (Liberty Aug-3, Braves Aug-10) arrived exactly this way and both carried negative CLV. (2) BOOK-INTEGRITY FLOOR: the order is void if Kalshi's two legs sum to 100c or less (e.g. NE 36c against SEA 64c). Our own conflict rule refuses a zero/negative synthetic hold on a degraded anchor, and an exchange showing one is showing a stale side, not a gift. Verified at compile: NE 39c + SEA 63c = 102c. PREMISES HELD AT COMPILE: Maye and Darnold both entirely absent from the injury report; NE C Ben Brown OUT. $15 at quarter-Kelly if filled at 37c (returns $41); ~$54 at 36c. || CANCELLED Wed 2026-09-09 12:01Z (8:01 AM ET, ~12h pre-kickoff), on the fallback wake. THE NAMED TRIGGER FIRED: TreVeyon Henderson was RULED OUT on New England's final injury report, released Tuesday Sep 8 - the exact condition clause (1) was written against. Market state at cancellation: Kalshi SEA 63c / NE 38c (sum 101c, so the book-integrity floor in clause (2) held). TWO SEPARATE FACTS, and they matter independently. FIRST: the order never filled on its own terms - 38c never reached the 37c trigger, so this is a no-fill regardless of the premise. SECOND: the market moved one cent IN OUR FAVOUR (39c -&gt; 38c, i.e. New England got cheaper), and that is exactly the trap the clause exists to catch - the price improved BECAUSE the true probability fell, not because value appeared. Had the drift carried one more cent to 37c we would have been handed a trigger print on a side whose premise had just deteriorated, which is the shape of both graded drift-fills (Liberty Aug-3, Braves Aug-10) that carried negative CLV. Standing the order down rather than leaving a resting trigger we would not honour. NOT RE-PRICED: a fresh fair would need a new compile, and this is a fallback wake, not a GO. At the compile fair the 38c price is -1.63% on the blend (+3.50% on the model alone), so nothing clears in any case.</t>
+          <t>HEADLINE ORDER - dispersion tier (+1.0% bar; Kalshi at 0.45 sharpness sits below the 0.50 fair-line floor, so it is a shop venue, never a fair source). Fires at 37c or better (2.7027, +170). Blended fair 2.675 (37.38%); the model ensemble alone says 39.33%, so a 37c fill is +1.03% on the blend and +6.30% on the model. Best live prices: BetRivers +160 (a fair source, so it carries the +1.5% model-tier bar = 2.715 and misses), Kalshi 39c = 2.5641. TWO BINDING CLAUSES. (1) DRIFT-CANCEL WITH A NAMED TRIGGER: TreVeyon Henderson (NE RB) has not practiced since Aug 24 and his final designation was still outstanding at compile. If New England reaches 37c ON A HENDERSON-OUT HEADLINE, that is a drift, not a fill - the premise our fair was built on changed, the true probability moved down with the price, and we stand down and re-price. A 37c print on ordinary two-way flow with no news is a legitimate standing-above fill. Both graded drift-fills (Liberty Aug-3, Braves Aug-10) arrived exactly this way and both carried negative CLV. (2) BOOK-INTEGRITY FLOOR: the order is void if Kalshi's two legs sum to 100c or less (e.g. NE 36c against SEA 64c). Our own conflict rule refuses a zero/negative synthetic hold on a degraded anchor, and an exchange showing one is showing a stale side, not a gift. Verified at compile: NE 39c + SEA 63c = 102c. PREMISES HELD AT COMPILE: Maye and Darnold both entirely absent from the injury report; NE C Ben Brown OUT. $15 at quarter-Kelly if filled at 37c (returns $41); ~$54 at 36c. || CANCELLED Wed 2026-09-09 12:01Z (8:01 AM ET, ~12h pre-kickoff), on the fallback wake. THE NAMED TRIGGER FIRED: TreVeyon Henderson was RULED OUT on New England's final injury report, released Tuesday Sep 8 - the exact condition clause (1) was written against. Market state at cancellation: Kalshi SEA 63c / NE 38c (sum 101c, so the book-integrity floor in clause (2) held). TWO SEPARATE FACTS, and they matter independently. FIRST: the order never filled on its own terms - 38c never reached the 37c trigger, so this is a no-fill regardless of the premise. SECOND: the market moved one cent IN OUR FAVOUR (39c -&gt; 38c, i.e. New England got cheaper), and that is exactly the trap the clause exists to catch - the price improved BECAUSE the true probability fell, not because value appeared. Had the drift carried one more cent to 37c we would have been handed a trigger print on a side whose premise had just deteriorated, which is the shape of both graded drift-fills (Liberty Aug-3, Braves Aug-10) that carried negative CLV. Standing the order down rather than leaving a resting trigger we would not honour. NOT RE-PRICED: a fresh fair would need a new compile, and this is a fallback wake, not a GO. At the compile fair the 38c price is -1.63% on the blend (+3.50% on the model alone), so nothing clears in any case. || SETTLED 2026-09-10. THREE FACTS, AND THEY DO NOT AGREE - recording all three. (1) NEVER FILLABLE. Kalshi's book sat 62 bid / 63 ask on Seattle all week, which is NE 37 BID / 38 ASK. Our 37c order was a bid joining the queue, not a takeable offer, and no source documents New England ever offered below 38c. So this was a no-fill on mechanics regardless of the cancel. (2) IT WOULD HAVE LOST. New England lost outright 13-10, so any fill loses the $15 stake. (3) AND YET IT GRADES AS A PROCESS MISS BY OUR OWN STANDARD. The close devigs to NE 0.3895; at 37c that is +5.28% no-vig CLV - by a wide margin the best CLV any order in this ledger has carried, against five prior fills that were ALL negative. Our doctrine says CLV, not P&amp;L, is the verdict. So: the price was right and we talked ourselves out of it. THE REASONING THAT FAILED: the drift-cancel clause assumed that if New England got cheaper after Henderson was ruled out, the price improved BECAUSE the true probability fell. That inference was testable and it was FALSE. The market moved toward New England all week - spread 3.5 -&gt; 3, DK ML -175 -&gt; -170 - which is precisely the convergence our own football module predicted when it devigged the spread to 3.29. We wrote a clause against news and it fired on a market correction our own model had already called. HYPOTHESIS PRE-REGISTERED, NOT ADOPTED (Walters rule, n=1): the drift-cancel test needs a second question - is the price moving AWAY from our model's number (real premise decay, stand down) or TOWARD it (the market agreeing with us, which is the opposite of a reason to cancel)? Needs more graded cases before it changes anything.</t>
         </is>
       </c>
     </row>
@@ -4648,7 +4650,7 @@
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>read right, thesis wrong - correctly declined</t>
         </is>
       </c>
       <c r="I76" s="5" t="n">
@@ -4663,12 +4665,12 @@
       </c>
       <c r="M76" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>worked</t>
         </is>
       </c>
       <c r="N76" s="2" t="inlineStr">
         <is>
-          <t>DECLINED READ, registered so it can be graded. Forecast for the 5:20-8:30 PM PT window at open-air Lumen: 20-30 mph gusts across the Puget Sound lowlands strengthening into the evening, plus moderate-to-heavy rain. That is a real under thesis and it is the most confident qualitative statement on this card. It is NOT BET for three independent reasons, any one of which is sufficient: totals never headline (standing rule); FanDuel and BookmakersReview both sit 44.5 -110/-110 with zero cross-venue dispersion, so there is no venue to buy it at; and we carry no calibrated weather model, so any probability we asserted would be invented. The ESPN listing's 45.5 would be the number to buy under if it were real, but it is one-sided and undated. Settle should record whether the game went under 44.5 - if this read keeps grading right while unpriced, that is evidence for building a weather layer, which is a parameter change and needs ledger evidence first.</t>
+          <t>DECLINED READ, registered so it can be graded. Forecast for the 5:20-8:30 PM PT window at open-air Lumen: 20-30 mph gusts across the Puget Sound lowlands strengthening into the evening, plus moderate-to-heavy rain. That is a real under thesis and it is the most confident qualitative statement on this card. It is NOT BET for three independent reasons, any one of which is sufficient: totals never headline (standing rule); FanDuel and BookmakersReview both sit 44.5 -110/-110 with zero cross-venue dispersion, so there is no venue to buy it at; and we carry no calibrated weather model, so any probability we asserted would be invented. The ESPN listing's 45.5 would be the number to buy under if it were real, but it is one-sided and undated. Settle should record whether the game went under 44.5 - if this read keeps grading right while unpriced, that is evidence for building a weather layer, which is a parameter change and needs ledger evidence first. || SETTLED 2026-09-10. THE UNDER CASHED BY 21.5 POINTS - 23 total against 44.5 - AND THE THESIS WAS WRONG. The forecast 20-30 mph gusts and heavy rain NEVER MATERIALIZED: actual conditions were winds under 6 mph, gusts topping out at 9, and zero precipitation, with DK Network stating flatly that weather had no impact on the game. The 23 points came from defense and turnovers - three fourth-quarter New England interceptions and a Seattle offense that was shut out in the first half after losing Darnold on the opening drive. So a bet placed on our stated reasoning would have won money for a reason that did not happen. THIS IS EVIDENCE AGAINST BUILDING A WEATHER LAYER, NOT FOR ONE - the read was right and the model behind it was wrong, which is the single most misleading way for a thesis to grade. Declining stays correct on all three original grounds (totals never headline; both books at 44.5 -110/-110 with no venue to buy it; no calibrated weather model). Logged loudly so a future cycle does not cite 'the Lumen under' as support for weather modelling.</t>
         </is>
       </c>
     </row>
@@ -4690,7 +4692,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I228"/>
+  <dimension ref="A1:I229"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -13377,6 +13379,44 @@
         </is>
       </c>
     </row>
+    <row r="229">
+      <c r="A229" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B229" s="2" t="inlineStr">
+        <is>
+          <t>nfl-2026-09-09-ne-sea</t>
+        </is>
+      </c>
+      <c r="C229" s="8" t="n">
+        <v>0.6262</v>
+      </c>
+      <c r="D229" s="8" t="n">
+        <v>0.6105</v>
+      </c>
+      <c r="E229" s="9">
+        <f>ABS(C229-D229)*100</f>
+        <v/>
+      </c>
+      <c r="F229" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G229" s="10">
+        <f>(C229-F229)^2</f>
+        <v/>
+      </c>
+      <c r="H229" s="10">
+        <f>(D229-F229)^2</f>
+        <v/>
+      </c>
+      <c r="I229" s="2" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -13388,7 +13428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B99"/>
+  <dimension ref="A1:B101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -13500,634 +13540,652 @@
     <row r="13">
       <c r="A13" s="13" t="inlineStr">
         <is>
-          <t>Open orders / pending</t>
+          <t>Orders cancelled (premise)</t>
         </is>
       </c>
       <c r="B13" s="14">
-        <f>COUNTIF(Bets!H:H,"pending")</f>
+        <f>COUNTIF(Bets!D:D,"order_cancelled")</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="13" t="inlineStr">
         <is>
-          <t>Decisions settled</t>
+          <t>Open orders / pending</t>
         </is>
       </c>
       <c r="B14" s="14">
-        <f>COUNTIF(Bets!M:M,"worked")+COUNTIF(Bets!M:M,"miss")</f>
+        <f>COUNTIF(Bets!H:H,"pending")</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="13" t="inlineStr">
         <is>
-          <t>Process validated (worked)</t>
+          <t>Decisions settled</t>
         </is>
       </c>
       <c r="B15" s="14">
-        <f>COUNTIF(Bets!M:M,"worked")</f>
+        <f>COUNTIF(Bets!M:M,"worked")+COUNTIF(Bets!M:M,"miss")</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="13" t="inlineStr">
         <is>
-          <t>Process misses</t>
+          <t>Process validated (worked)</t>
         </is>
       </c>
       <c r="B16" s="14">
-        <f>COUNTIF(Bets!M:M,"miss")</f>
+        <f>COUNTIF(Bets!M:M,"worked")</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="13" t="inlineStr">
         <is>
-          <t>Fair lines graded</t>
+          <t>Process misses</t>
         </is>
       </c>
       <c r="B17" s="14">
-        <f>COUNT(FairLines!E:E)</f>
+        <f>COUNTIF(Bets!M:M,"miss")</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="13" t="inlineStr">
         <is>
-          <t>Mean |fair − close| (pts)</t>
-        </is>
-      </c>
-      <c r="B18" s="18">
-        <f>IFERROR(AVERAGE(FairLines!E:E),0)</f>
+          <t>Fair lines graded</t>
+        </is>
+      </c>
+      <c r="B18" s="14">
+        <f>COUNT(FairLines!E:E)</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="13" t="inlineStr">
         <is>
-          <t>Max |fair − close| (pts)</t>
+          <t>Mean |fair − close| (pts)</t>
         </is>
       </c>
       <c r="B19" s="18">
-        <f>IFERROR(MAX(FairLines!E:E),0)</f>
+        <f>IFERROR(AVERAGE(FairLines!E:E),0)</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="13" t="inlineStr">
         <is>
-          <t>Clean-source mean error (pts)</t>
+          <t>Max |fair − close| (pts)</t>
         </is>
       </c>
       <c r="B20" s="18">
-        <f>IFERROR(AVERAGEIFS(FairLines!E:E,FairLines!I:I,"clean"),0)</f>
+        <f>IFERROR(MAX(FairLines!E:E),0)</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="13" t="inlineStr">
         <is>
-          <t>Flagged-source mean error (pts)</t>
+          <t>Clean-source mean error (pts)</t>
         </is>
       </c>
       <c r="B21" s="18">
-        <f>IFERROR(AVERAGEIFS(FairLines!E:E,FairLines!I:I,"&lt;&gt;clean"),0)</f>
+        <f>IFERROR(AVERAGEIFS(FairLines!E:E,FairLines!I:I,"clean"),0)</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="13" t="inlineStr">
         <is>
-          <t>Brier — SharpOds fair</t>
-        </is>
-      </c>
-      <c r="B22" s="19">
-        <f>IFERROR(AVERAGE(FairLines!G:G),0)</f>
+          <t>Flagged-source mean error (pts)</t>
+        </is>
+      </c>
+      <c r="B22" s="18">
+        <f>IFERROR(AVERAGEIFS(FairLines!E:E,FairLines!I:I,"&lt;&gt;clean"),0)</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="13" t="inlineStr">
         <is>
-          <t>Brier — closing line</t>
+          <t>Brier — SharpOds fair</t>
         </is>
       </c>
       <c r="B23" s="19">
-        <f>IFERROR(AVERAGE(FairLines!H:H),0)</f>
+        <f>IFERROR(AVERAGE(FairLines!G:G),0)</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="13" t="inlineStr">
         <is>
+          <t>Brier — closing line</t>
+        </is>
+      </c>
+      <c r="B24" s="19">
+        <f>IFERROR(AVERAGE(FairLines!H:H),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
           <t>Brier — coin flip (reference)</t>
         </is>
       </c>
-      <c r="B24" s="19">
+      <c r="B25" s="19">
         <f>0.25</f>
         <v/>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="20" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="20" t="inlineStr">
         <is>
           <t>What worked / what didn't (from the decision log)</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="21" t="inlineStr">
-        <is>
-          <t>[WORKED] Full 5-game slate: Favorites went 2-3; both most-likely sides blew 6+ run leads; every listed price was -EV vs fair (avg -3.3%). Passing saved money.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] BAL @ DET: Line closed 1.56-1.59, moving away; discipline held. Tigers lost 9-10 in 12 - a chased fill would have lost.</t>
+          <t>[WORKED] Full 5-game slate: Favorites went 2-3; both most-likely sides blew 6+ run leads; every listed price was -EV vs fair (avg -3.3%). Passing saved money.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] CHC @ STL: Labeled unverified staleness and not executed; the close proved it was quote drift, not free money.</t>
+          <t>[WORKED] BAL @ DET: Line closed 1.56-1.59, moving away; discipline held. Tigers lost 9-10 in 12 - a chased fill would have lost.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] NYY @ CHC: Close CHC -140 landed on the sportsbook consensus; Polymarket 52c was the stale outlier (NYY won 2-0 as a +130 dog - vs the close that bet was -7% EV luck). Refusal correct.</t>
+          <t>[WORKED] CHC @ STL: Labeled unverified staleness and not executed; the close proved it was quote drift, not free money.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] PHI @ BAL: PHI never traded above 2.06 (target 2.10). Close no-vig PHI 0.467: even at target the bet was -2% vs close - not filling saved money. SportsGrid model lean (PHI 54%) was the wrong side per the close.</t>
+          <t>[WORKED] NYY @ CHC: Close CHC -140 landed on the sportsbook consensus; Polymarket 52c was the stale outlier (NYY won 2-0 as a +130 dog - vs the close that bet was -7% EV luck). Refusal correct.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] PIT @ CIN: PIT -120 to -136 all day, never near the 1.966 target. Close no-vig PIT 0.564: a 1.966 fill would have been ~+11% EV vs close - right side, market never paid the price.</t>
+          <t>[WORKED] PHI @ BAL: PHI never traded above 2.06 (target 2.10). Close no-vig PHI 0.467: even at target the bet was -2% vs close - not filling saved money. SportsGrid model lean (PHI 54%) was the wrong side per the close.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] PIT @ CIN: CIN never traded above +106 (2.06) - 17 cents short of the 2.231 bar; the '+120 one source' quote was never corroborated. CIN lost 1-4, so no fill dodged a loss; vs the no-vig close a 2.231 fill would still have been +EV (right side, market never paid).</t>
+          <t>[WORKED] PIT @ CIN: PIT -120 to -136 all day, never near the 1.966 target. Close no-vig PIT 0.564: a 1.966 fill would have been ~+11% EV vs close - right side, market never paid the price.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] NYY @ CHC: Refusal correct, with a twist: the close landed NYY road-favorite (-122 to -132; CHC +102/+105) - the OPPOSITE of our 'books CHC 1.62' quote, which no closing book corroborates. That quote was stale/wrong (flagged for provenance). Polymarket NYY 54c was actually the consensus side. CHC won 5-2 anyway - neither side's value story survived. Conflict rule worked for the right reason: garbage inputs were refused, not priced.</t>
+          <t>[WORKED] PIT @ CIN: CIN never traded above +106 (2.06) - 17 cents short of the 2.231 bar; the '+120 one source' quote was never corroborated. CIN lost 1-4, so no fill dodged a loss; vs the no-vig close a 2.231 fill would still have been +EV (right side, market never paid).</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] WSH @ ATL: Braves 8-3. Polymarket-only board stayed unpriced per the 0.45-sharpness demotion; no book close collected for this game.</t>
+          <t>[WORKED] NYY @ CHC: Refusal correct, with a twist: the close landed NYY road-favorite (-122 to -132; CHC +102/+105) - the OPPOSITE of our 'books CHC 1.62' quote, which no closing book corroborates. That quote was stale/wrong (flagged for provenance). Polymarket NYY 54c was actually the consensus side. CHC won 5-2 anyway - neither side's value story survived. Conflict rule worked for the right reason: garbage inputs were refused, not priced.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] PHI @ BAL: Fill ambiguous: consensus close +119 (2.19) never reached the 2.225 bar, but SportsGrid reported 'BAL +125 at other books' pregame, which would have filled. Graded no-fill on the consensus board we price from. BAL lost 0-5, so neither grading forfeits a win; a phantom fill would have lost. Single-book-anchor caveat from pre-registration stands.</t>
+          <t>[WORKED] WSH @ ATL: Braves 8-3. Polymarket-only board stayed unpriced per the 0.45-sharpness demotion; no book close collected for this game.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] SEA @ POR (MLS): NO BET - user report (the only fill oracle; pages 403 post-hoc): the prediction-market ask had moved above the 45c stand-down line (engine minimum 2.23) by bet time, so per the slip's own fill rule the order did not fire. Paper grade of the 2.273 listed snapshot: Portland won 2-1 and the number beat the bet365 close 2.05/3.80/3.00 by +10.9% raw / +4.5% no-vig - the edge was real at the snapshot, and it decayed before execution. Standing down was correct: at the moved ask the +2.5% EV bar was no longer met.</t>
+          <t>[WORKED] PHI @ BAL: Fill ambiguous: consensus close +119 (2.19) never reached the 2.225 bar, but SportsGrid reported 'BAL +125 at other books' pregame, which would have filled. Graded no-fill on the consensus board we price from. BAL lost 0-5, so neither grading forfeits a win; a phantom fill would have lost. Single-book-anchor caveat from pre-registration stands.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] PIT @ CIN: Refusal validated on PROCESS: the book-vs-Polymarket gap (CIN 1.676 vs 55c) never visibly converged before first pitch - the market stayed unpriceable by our rule at every observable snapshot. CIN won 10-2 (Burns 6 IP 9 K) and the close landed -148, but outcome isn't the verdict; the conflict rule is now 4-for-4 on process. Pre-registered under the conflict rule, graded at the close.</t>
+          <t>[WORKED] SEA @ POR (MLS): NO BET - user report (the only fill oracle; pages 403 post-hoc): the prediction-market ask had moved above the 45c stand-down line (engine minimum 2.23) by bet time, so per the slip's own fill rule the order did not fire. Paper grade of the 2.273 listed snapshot: Portland won 2-1 and the number beat the bet365 close 2.05/3.80/3.00 by +10.9% raw / +4.5% no-vig - the edge was real at the snapshot, and it decayed before execution. Standing down was correct: at the moved ask the +2.5% EV bar was no longer met.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] STL @ NYY (7:05 PM ET Mon): NOT FILLED - and saved by it. Every dated Monday price moved AWAY from the 1.599 trigger (NYY -186 Sunday -&gt; -195/-210/-217/-235 across books at close); then NYY lost 7-13 (Burleson 3 HR off Schlittler). Our fair (64.1%) sat above a close (~65%) that the result embarrassed - calibration fine, outcome brutal, order discipline kept the stake at zero.</t>
+          <t>[WORKED] PIT @ CIN: Refusal validated on PROCESS: the book-vs-Polymarket gap (CIN 1.676 vs 55c) never visibly converged before first pitch - the market stayed unpriceable by our rule at every observable snapshot. CIN won 10-2 (Burns 6 IP 9 K) and the close landed -148, but outcome isn't the verdict; the conflict rule is now 4-for-4 on process. Pre-registered under the conflict rule, graded at the close.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] SFG @ TEX (8:05 PM ET Mon): NOT FILLED - TEX never reached plus-money (observed -105 to -125 across books; +103 trigger unreached), then lost 1-5 with five errors behind Webb's 6 shutout IP. Second unfilled loser dodged on the day.</t>
+          <t>[WORKED] STL @ NYY (7:05 PM ET Mon): NOT FILLED - and saved by it. Every dated Monday price moved AWAY from the 1.599 trigger (NYY -186 Sunday -&gt; -195/-210/-217/-235 across books at close); then NYY lost 7-13 (Burleson 3 HR off Schlittler). Our fair (64.1%) sat above a close (~65%) that the result embarrassed - calibration fine, outcome brutal, order discipline kept the stake at zero.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] SDP @ AZ (9:40 PM ET Mon): Rejection fully validated: the real Monday market was near pick'em with ARI a slight HOME favorite (BetMGM/DK SDP -102 / ARI -118; Yahoo -113) - the garbled 'SD -185/ARI +737' board was wrong on side AND magnitude. ARI won 5-1. Garbage in, nothing out: correct.</t>
+          <t>[WORKED] SFG @ TEX (8:05 PM ET Mon): NOT FILLED - TEX never reached plus-money (observed -105 to -125 across books; +103 trigger unreached), then lost 1-5 with five errors behind Webb's 6 shutout IP. Second unfilled loser dodged on the day.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] ATH @ CIN (start time unverified; typical 12:35 PM ET getaway): NOT FILLED: CIN drifted our way (-171 open -&gt; -158 at first pitch) but never reached the -147 (1.679) bar; best documented 1.633. CIN won 6-5, and a 1.679 fill would have carried +2.8% raw CLV vs the close - right side, right price demand, market never paid it. Reverse line movement toward the road dog noted pregame; the bar held anyway.</t>
+          <t>[WORKED] SDP @ AZ (9:40 PM ET Mon): Rejection fully validated: the real Monday market was near pick'em with ARI a slight HOME favorite (BetMGM/DK SDP -102 / ARI -118; Yahoo -113) - the garbled 'SD -185/ARI +737' board was wrong on side AND magnitude. ARI won 5-1. Garbage in, nothing out: correct.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] Dinamo Minsk @ Braga (UECL Q3 leg 1; kickoff ~3:00-3:45 PM ET assumed): NOT FILLED: Braga sat 1.10-1.11 everywhere pre-match; the 1.141 re-verified quote never existed. Braga won 1-0. The demotion logic validated exactly: on extreme favorites the only 'fills' available are cross-book noise, and even that noise stayed under 4 cents.</t>
+          <t>[WORKED] ATH @ CIN (start time unverified; typical 12:35 PM ET getaway): NOT FILLED: CIN drifted our way (-171 open -&gt; -158 at first pitch) but never reached the -147 (1.679) bar; best documented 1.633. CIN won 6-5, and a 1.679 fill would have carried +2.8% raw CLV vs the close - right side, right price demand, market never paid it. Reverse line movement toward the road dog noted pregame; the bar held anyway.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] ARI @ CAR, Hall of Fame Game (8:00 PM ET Thu, Canton - neutral site): NOT FILLED by one cent of juice: ARI +1.5 reached ~-115 game-day vs the -114 bar - and then LOST (CAR won by exactly 3 on the final play). The near-miss dodged a loser; fill discipline is net positive on the card (two would-have-won fills never reached target, the one would-have-lost fill missed by a cent).</t>
+          <t>[WORKED] Dinamo Minsk @ Braga (UECL Q3 leg 1; kickoff ~3:00-3:45 PM ET assumed): NOT FILLED: Braga sat 1.10-1.11 everywhere pre-match; the 1.141 re-verified quote never existed. Braga won 1-0. The demotion logic validated exactly: on extreme favorites the only 'fills' available are cross-book noise, and even that noise stayed under 4 cents.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] ARI @ CAR (HOF Game): Suppression validated on process with an ironic outcome: the suppressed leg (ARI +1.5 -&gt; +7.5) would have back-doored a win (lost by 3), but the game produced 63 points against a 34.5 total - preseason margins have NO key-number structure, which is precisely why the leg had no business existing. Note-only; engine gating change still deferred (Walters rule).</t>
+          <t>[WORKED] ARI @ CAR, Hall of Fame Game (8:00 PM ET Thu, Canton - neutral site): NOT FILLED by one cent of juice: ARI +1.5 reached ~-115 game-day vs the -114 bar - and then LOST (CAR won by exactly 3 on the final play). The near-miss dodged a loser; fill discipline is net positive on the card (two would-have-won fills never reached target, the one would-have-lost fill missed by a cent).</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] Shnaider vs Swiatek, WTA Toronto QF (7:00 PM ET Mon): NOT FILLED: no book ever printed 1.403+ (-285/-300 everywhere). Swiatek won 6-2 6-1 - a missed winner, which is the cost side of the same discipline that has dodged three losers. The bar cuts both ways; that is the design.</t>
+          <t>[WORKED] ARI @ CAR (HOF Game): Suppression validated on process with an ironic outcome: the suppressed leg (ARI +1.5 -&gt; +7.5) would have back-doored a win (lost by 3), but the game produced 63 points against a 34.5 total - preseason margins have NO key-number structure, which is precisely why the leg had no business existing. Note-only; engine gating change still deferred (Walters rule).</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] COL @ AZ (Chase Field, evening - exact time TBC): NOT FILLED: line moved AWAY from the order all day (-179 -&gt; -190s; the -164 outlier board never reached -160). Game in progress at grading - outcome irrelevant to an unfilled order.</t>
+          <t>[WORKED] Shnaider vs Swiatek, WTA Toronto QF (7:00 PM ET Mon): NOT FILLED: no book ever printed 1.403+ (-285/-300 everywhere). Swiatek won 6-2 6-1 - a missed winner, which is the cost side of the same discipline that has dodged three losers. The bar cuts both ways; that is the design.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] KC @ LAD (10:10 PM ET Mon - Skubal home debut): VALIDATED, with the sharpest twist yet: the definitive Monday close was LAD -325/-330 (FanDuel + 'other oddsmakers' + Polymarket 74c all agree near 76%) - the -160 board we saw was itself a stale/erroneous print. The conflict was real, and this time the BOOK leg was the garbage and the prediction market was near truth (mirror of the Aug-1 stale 'CHC 1.62'). The rule doesn't care which source lies - it refuses the disagreement. LAD needed a 7th-inning rally to win 6-5. 7-for-7 on refusals/flags.</t>
+          <t>[WORKED] COL @ AZ (Chase Field, evening - exact time TBC): NOT FILLED: line moved AWAY from the order all day (-179 -&gt; -190s; the -164 outlier board never reached -160). Game in progress at grading - outcome irrelevant to an unfilled order.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] CLE @ DET (6:40 PM ET Tue, Comerica): NOT FILLED - the market ran the other way, hard: DET +113 Monday night -&gt; -120/-121 favorite at first pitch. No +116 ever printed. DET won 6-4, so another would-have-won missed - but the swing's SIZE is the lesson: an overnight board can embed a different starting pitcher than game-day reality (Drew Anderson started). Listed-pitcher rule: every future order names its assumed starters, and a change voids the premise (Skenes-scratch lesson, Jul 30, finally codified).</t>
+          <t>[WORKED] KC @ LAD (10:10 PM ET Mon - Skubal home debut): VALIDATED, with the sharpest twist yet: the definitive Monday close was LAD -325/-330 (FanDuel + 'other oddsmakers' + Polymarket 74c all agree near 76%) - the -160 board we saw was itself a stale/erroneous print. The conflict was real, and this time the BOOK leg was the garbage and the prediction market was near truth (mirror of the Aug-1 stale 'CHC 1.62'). The rule doesn't care which source lies - it refuses the disagreement. LAD needed a 7th-inning rally to win 6-5. 7-for-7 on refusals/flags.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] TB @ ATH (9:40 PM ET Tue): NOT FILLED - TB shortened -146 -&gt; -180 and won 12-4. Fourth straight unfilled order whose side won. Tempting to call the bar too high; the ledger says otherwise - the only two orders that DID fill both carried negative CLV and went 1-1. Unfilled winners are the visible cost of refusing bad prices; filled losers are the invisible cost of chasing. No parameter change (Walters rule).</t>
+          <t>[WORKED] CLE @ DET (6:40 PM ET Tue, Comerica): NOT FILLED - the market ran the other way, hard: DET +113 Monday night -&gt; -120/-121 favorite at first pitch. No +116 ever printed. DET won 6-4, so another would-have-won missed - but the swing's SIZE is the lesson: an overnight board can embed a different starting pitcher than game-day reality (Drew Anderson started). Listed-pitcher rule: every future order names its assumed starters, and a change voids the premise (Skenes-scratch lesson, Jul 30, finally codified).</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] KC @ LAD (10:10 PM ET Tue): Book LAD -285 vs Polymarket 72c: nearly agreeing today, but cross-source best prices still net -0.99% hold - the rule is binary and fires the same on small conflicts as wide ones (that binariness is the Cubs-3.7pt lesson). 6th application. Monday's refusal grades at its close next cycle alongside this one. || SETTLED: close LAD -275 (~70-71% no-vig) vs Polymarket 72c - the sources converged AT the close, meaning no exploitable edge ever existed. LAD won 5-4. Refusals now 8-for-8.</t>
+          <t>[WORKED] TB @ ATH (9:40 PM ET Tue): NOT FILLED - TB shortened -146 -&gt; -180 and won 12-4. Fourth straight unfilled order whose side won. Tempting to call the bar too high; the ledger says otherwise - the only two orders that DID fill both carried negative CLV and went 1-1. Unfilled winners are the visible cost of refusing bad prices; filled losers are the invisible cost of chasing. No parameter change (Walters rule).</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] NYM @ ATL (7:15 PM ET Wed; PITCHERS: Thornton vs Mahle): NOT FILLED - the board moved the wrong way all day (-156 -&gt; -158/-175 close); -150 never printed. ATL won 6-3: the FIFTH straight unfilled order whose side won. Pattern reading: our fairs are directionally right and the market agrees too fast to pay our price - which is what near-parity Brier with the close predicts. The bar stays (Walters rule); the edge has to come from being earlier, not looser.</t>
+          <t>[WORKED] KC @ LAD (10:10 PM ET Tue): Book LAD -285 vs Polymarket 72c: nearly agreeing today, but cross-source best prices still net -0.99% hold - the rule is binary and fires the same on small conflicts as wide ones (that binariness is the Cubs-3.7pt lesson). 6th application. Monday's refusal grades at its close next cycle alongside this one. || SETTLED: close LAD -275 (~70-71% no-vig) vs Polymarket 72c - the sources converged AT the close, meaning no exploitable edge ever existed. LAD won 5-4. Refusals now 8-for-8.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] ATP Montreal SF: Jodar vs Nakashima (6:00 PM ET Wed): FILL CONDITION MET VIA CROSS-BOOK SHOPPING - AND WON. +200 (&gt;= the +197 trigger) was genuinely available at a book pre-match while Dimers' board showed +188; Nakashima won 7-6(3) 6-4. At the 2.969 floor vs the 2.94 close: raw CLV +1.0%, no-vig -1.7% - the first fill in this ledger with POSITIVE RAW CLV and the best fill-CLV recorded (prior fills: -5.4% and -3.1% no-vig), precisely because it came from price dispersion across books (allowed) rather than line drift (forbidden). The drift-vs-shopping distinction now has favorable evidence on the shopping side. Paper grade, stake 0 - backup order, user bets headline only.</t>
+          <t>[WORKED] NYM @ ATL (7:15 PM ET Wed; PITCHERS: Thornton vs Mahle): NOT FILLED - the board moved the wrong way all day (-156 -&gt; -158/-175 close); -150 never printed. ATL won 6-3: the FIFTH straight unfilled order whose side won. Pattern reading: our fairs are directionally right and the market agrees too fast to pay our price - which is what near-parity Brier with the close predicts. The bar stays (Walters rule); the edge has to come from being earlier, not looser.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] SEA @ NYY (7:05 PM ET Wed; PITCHERS: Miller vs Warren): NOT FILLED - opened -119 and firmed to -131; the -112 trigger never printed. NYY won 10-5 anyway (sixth unfilled winner if you count this one alongside the ATL streak).</t>
+          <t>[WORKED] ATP Montreal SF: Jodar vs Nakashima (6:00 PM ET Wed): FILL CONDITION MET VIA CROSS-BOOK SHOPPING - AND WON. +200 (&gt;= the +197 trigger) was genuinely available at a book pre-match while Dimers' board showed +188; Nakashima won 7-6(3) 6-4. At the 2.969 floor vs the 2.94 close: raw CLV +1.0%, no-vig -1.7% - the first fill in this ledger with POSITIVE RAW CLV and the best fill-CLV recorded (prior fills: -5.4% and -3.1% no-vig), precisely because it came from price dispersion across books (allowed) rather than line drift (forbidden). The drift-vs-shopping distinction now has favorable evidence on the shopping side. Paper grade, stake 0 - backup order, user bets headline only.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] MIL @ LAD (10:10 PM ET Thu; PITCHERS: Drohan vs Sasaki): NOT FILLED - EdgeBets' 8-book closing recap tops MIL out at +129 (range +115/+129, consensus +123/+125); the +136 trigger never printed anywhere. Both listed pitchers started (Shane Drohan vs Sasaki) so the premise held; the price just never came. MIL won 5-4 on a 3-run 9th - the SEVENTH unfilled order whose side won. The bar stays (Walters rule): the two orders that ever DID fill via drift carried the ledger's worst CLV.</t>
+          <t>[WORKED] SEA @ NYY (7:05 PM ET Wed; PITCHERS: Miller vs Warren): NOT FILLED - opened -119 and firmed to -131; the -112 trigger never printed. NYY won 10-5 anyway (sixth unfilled winner if you count this one alongside the ATL streak).</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] PHI @ MIN, Field of Dreams (7:30 PM ET; Nola vs Bradley; RAIN RISK): NOT FILLED - Over sat -118/-120 all day and never reached the -107 trigger. Game went UNDER (8 runs): the FIRST unfilled order whose side LOST, i.e. the bar's first visible counterfactual save (~$40 at quarter-Kelly). The unfilled-order ledger is now 7 winners, 1 loser - and the loser is the one the bar refused to pay for. First graded third-party total model (SportsLine 60.2% over): WRONG. Rain clause never triggered - played as scheduled.</t>
+          <t>[WORKED] MIL @ LAD (10:10 PM ET Thu; PITCHERS: Drohan vs Sasaki): NOT FILLED - EdgeBets' 8-book closing recap tops MIL out at +129 (range +115/+129, consensus +123/+125); the +136 trigger never printed anywhere. Both listed pitchers started (Shane Drohan vs Sasaki) so the premise held; the price just never came. MIL won 5-4 on a 3-run 9th - the SEVENTH unfilled order whose side won. The bar stays (Walters rule): the two orders that ever DID fill via drift carried the ledger's worst CLV.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] PHI @ MIN, Field of Dreams (same game): NOT FILLED - PHI ranged -102/-104 all day and closed ~-103 (SBR); the +106 trigger needed plus-money that never printed. PHI won 7-1 (Schwarber 2 HR) - the EIGHTH unfilled order graded, 7 of whose sides won.</t>
+          <t>[WORKED] PHI @ MIN, Field of Dreams (7:30 PM ET; Nola vs Bradley; RAIN RISK): NOT FILLED - Over sat -118/-120 all day and never reached the -107 trigger. Game went UNDER (8 runs): the FIRST unfilled order whose side LOST, i.e. the bar's first visible counterfactual save (~$40 at quarter-Kelly). The unfilled-order ledger is now 7 winners, 1 loser - and the loser is the one the bar refused to pay for. First graded third-party total model (SportsLine 60.2% over): WRONG. Rain clause never triggered - played as scheduled.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] KC @ LAA (9:38 PM ET Sat; PITCHERS: Dobnak vs Detmers): NOT FILLED - KC never evidenced past +135 (trigger +147) and Polymarket sat pinned at the 41c board price all day; no 40.5c ask printed. Fill oracle open: if your execution says otherwise, report and I regrade. COUNTERFACTUAL SAVE #2, and the biggest yet: KC was SHUT OUT 1-0 (Detmers 8 scoreless, 11 K). The closest-to-live order in ledger history would have lost at any fill price. Dobnak/Detmers premise held.</t>
+          <t>[WORKED] PHI @ MIN, Field of Dreams (same game): NOT FILLED - PHI ranged -102/-104 all day and closed ~-103 (SBR); the +106 trigger needed plus-money that never printed. PHI won 7-1 (Schwarber 2 HR) - the EIGHTH unfilled order graded, 7 of whose sides won.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] SD @ CLE (7:10 PM ET Sat; ASSUMED pitchers Vasquez-SD vs Cantillo-CLE, side-assignment UNVERIFIED): VOID ON THE PREMISE CLAUSE, and unfilled anyway: San Diego ran a Wandy Peralta OPENER instead of listed probable Vasquez (Cantillo did start for CLE), and the written clause - 'void unless the pairing is confirmed at bet time' - fired exactly as designed. The price also ran away (+118 -&gt; +105, never +127). SD lost 6-1: save #3 on the same card.</t>
+          <t>[WORKED] KC @ LAA (9:38 PM ET Sat; PITCHERS: Dobnak vs Detmers): NOT FILLED - KC never evidenced past +135 (trigger +147) and Polymarket sat pinned at the 41c board price all day; no 40.5c ask printed. Fill oracle open: if your execution says otherwise, report and I regrade. COUNTERFACTUAL SAVE #2, and the biggest yet: KC was SHUT OUT 1-0 (Detmers 8 scoreless, 11 K). The closest-to-live order in ledger history would have lost at any fill price. Dobnak/Detmers premise held.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] STL @ CHC (2:20 PM ET Sat; PITCHERS: McGreevy vs Boyd): NOT FILLED - CHC shortened hard from -166 to -174/-185 closes; -149 never printed. McGreevy/Boyd started as listed - and Boyd (8-1) was tagged for three Baez HRs in an 8-4 loss. Save #4... third of THREE on this card alone. Every Saturday order's side lost; the bar refused all of them.</t>
+          <t>[WORKED] SD @ CLE (7:10 PM ET Sat; ASSUMED pitchers Vasquez-SD vs Cantillo-CLE, side-assignment UNVERIFIED): VOID ON THE PREMISE CLAUSE, and unfilled anyway: San Diego ran a Wandy Peralta OPENER instead of listed probable Vasquez (Cantillo did start for CLE), and the written clause - 'void unless the pairing is confirmed at bet time' - fired exactly as designed. The price also ran away (+118 -&gt; +105, never +127). SD lost 6-1: save #3 on the same card.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] SEA @ MIL (7:40 PM ET Tue, American Family Field; PITCHERS: Miller vs Harrison): NOT FILLED - the trigger was -131 or better and the market moved the WRONG way from the first print: -148 early -&gt; -150 open -&gt; -159/-160/-165 -&gt; -168 close. No book ever came within 17 cents of the trigger; no drift-through, so no re-price question. MIL then won 22-0, so the side won - but the close (61.6% no-vig) steamed PAST our 58.2% fair, meaning even a -148 take would have been the slow side of a sharp move our own model layer (60.7% MIL) partly anticipated. CORRECTED RUNNING TALLY of every order that never filled (incl. the voided SD premise): sides are now 9W-4L across 13 (Swiatek, CIN, DET, TB, ATL, NYY, MIL 8/13, PHI 8/13, MIL 8/18 won; FoD Over, KC, CHC, SD lost) - earlier notes' 7W counts undercounted by one, fixed here. Fill oracle stands: report an execution and I regrade.</t>
+          <t>[WORKED] STL @ CHC (2:20 PM ET Sat; PITCHERS: McGreevy vs Boyd): NOT FILLED - CHC shortened hard from -166 to -174/-185 closes; -149 never printed. McGreevy/Boyd started as listed - and Boyd (8-1) was tagged for three Baez HRs in an 8-4 loss. Save #4... third of THREE on this card alone. Every Saturday order's side lost; the bar refused all of them.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] Mirassol @ LDU Quito, Libertadores R16 leg 2 (6:00 PM ET Thu, Quito, 2850m; agg 1-1): NOT FILLED - no named book was ever pinned at 1.682+ (an unattributed ESPN-visible -145 = 1.690 existed but Pinnacle sat 1.55 simultaneously; the live-single-book-only condition was written for exactly this). COUNTERFACTUAL SAVE #5: the 90-min result was 0-0 - a fill would have LOST even as LDU advanced on penalties. Pricing lesson logged: the 1.60 averaged anchor sat between a 1.55 sharp and a 1.69 soft quote, so the order's 'edge' was partly anchor softness - averaged trios stay consensus-c and live-only forever. Never-filled sides: 9W-5L at this point in the pass.</t>
+          <t>[WORKED] SEA @ MIL (7:40 PM ET Tue, American Family Field; PITCHERS: Miller vs Harrison): NOT FILLED - the trigger was -131 or better and the market moved the WRONG way from the first print: -148 early -&gt; -150 open -&gt; -159/-160/-165 -&gt; -168 close. No book ever came within 17 cents of the trigger; no drift-through, so no re-price question. MIL then won 22-0, so the side won - but the close (61.6% no-vig) steamed PAST our 58.2% fair, meaning even a -148 take would have been the slow side of a sharp move our own model layer (60.7% MIL) partly anticipated. CORRECTED RUNNING TALLY of every order that never filled (incl. the voided SD premise): sides are now 9W-4L across 13 (Swiatek, CIN, DET, TB, ATL, NYY, MIL 8/13, PHI 8/13, MIL 8/18 won; FoD Over, KC, CHC, SD lost) - earlier notes' 7W counts undercounted by one, fixed here. Fill oracle stands: report an execution and I regrade.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] Dream @ Sparks, WNBA (10:00 PM ET Thu, Crypto.com Arena): VOID ON THE PREMISE CLAUSE, pre-game and result-independent: Brionna Jones was ruled OUT for the Dream (left leg, third straight miss) on final injury reports dated to this game - the pre-registered condition 'void if B. Jones or Reese is OUT' fired exactly as written. (Reese played; the 'questionable' chatter traced to July articles and was discarded on date discipline.) Second premise-clause void in a week (SD Padres opener was the first) - the clause class is earning its keep. No stake, no fill, no grade.</t>
+          <t>[WORKED] Mirassol @ LDU Quito, Libertadores R16 leg 2 (6:00 PM ET Thu, Quito, 2850m; agg 1-1): NOT FILLED - no named book was ever pinned at 1.682+ (an unattributed ESPN-visible -145 = 1.690 existed but Pinnacle sat 1.55 simultaneously; the live-single-book-only condition was written for exactly this). COUNTERFACTUAL SAVE #5: the 90-min result was 0-0 - a fill would have LOST even as LDU advanced on penalties. Pricing lesson logged: the 1.60 averaged anchor sat between a 1.55 sharp and a 1.69 soft quote, so the order's 'edge' was partly anchor softness - averaged trios stay consensus-c and live-only forever. Never-filled sides: 9W-5L at this point in the pass.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] 49ers @ Chargers, NFL preseason Wk 2 (10:00 PM ET Thu, SoFi): NOT FILLED on post-ship evidence - SF only SHORTENED after our card (board 1.769 -&gt; DK close 1.80... vs LAC flipping to dog the line moved through -118 to -125; an SF +102 quote exists but traces to early-week, pre-card). No post-ship 1.879+ at a named book evidenced; fill oracle open. SF won 41-17 - a would-have-won missed at the bar's usual price of discipline.</t>
+          <t>[WORKED] Dream @ Sparks, WNBA (10:00 PM ET Thu, Crypto.com Arena): VOID ON THE PREMISE CLAUSE, pre-game and result-independent: Brionna Jones was ruled OUT for the Dream (left leg, third straight miss) on final injury reports dated to this game - the pre-registered condition 'void if B. Jones or Reese is OUT' fired exactly as written. (Reese played; the 'questionable' chatter traced to July articles and was discarded on date discipline.) Second premise-clause void in a week (SD Padres opener was the first) - the clause class is earning its keep. No stake, no fill, no grade.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] America @ Juarez, Liga MX J5 (11:00 PM ET Fri, Estadio Olimpico Benito Juarez): NOT FILLED - the 1.945 trigger sat above the ENTIRE market all day (best anywhere: a 1.85 aggregate leg; consensus close ~1.76-1.77) and the market shortened toward America, who won 2-1. A would-have-won at a price that never existed - the bar's usual cost. Our Codere 1.82 anchor graded honest (slightly above close); the scary Bet365 -241 capture from Friday night was a bad aggregator read, not the market.</t>
+          <t>[WORKED] 49ers @ Chargers, NFL preseason Wk 2 (10:00 PM ET Thu, SoFi): NOT FILLED on post-ship evidence - SF only SHORTENED after our card (board 1.769 -&gt; DK close 1.80... vs LAC flipping to dog the line moved through -118 to -125; an SF +102 quote exists but traces to early-week, pre-card). No post-ship 1.879+ at a named book evidenced; fill oracle open. SF won 41-17 - a would-have-won missed at the bar's usual price of discipline.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] Coventry @ Arsenal, EPL opener (3:00 PM ET Fri, Emirates): NOT FILLED - best named-book price all day was DK -475 (1.211); the 1.224 trigger never printed (FanDuel closed -550). Arsenal won 3-0: a would-have-won that never offered the price. The extreme-favorite demotion was correct: the market's ceiling sat below our bar all day.</t>
+          <t>[WORKED] America @ Juarez, Liga MX J5 (11:00 PM ET Fri, Estadio Olimpico Benito Juarez): NOT FILLED - the 1.945 trigger sat above the ENTIRE market all day (best anywhere: a 1.85 aggregate leg; consensus close ~1.76-1.77) and the market shortened toward America, who won 2-1. A would-have-won at a price that never existed - the bar's usual cost. Our Codere 1.82 anchor graded honest (slightly above close); the scary Bet365 -241 capture from Friday night was a bad aggregator read, not the market.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] Coventry @ Arsenal, same match - total 2.5: NOT FILLED - Over 2.5 closed -176/-181 (1.552-1.568); the 1.662 trigger never evidenced. It landed (3 goals) and SportsLine's 64% graded RIGHT on its first EPL outing - a model note for the file, priced away by the market. Never-filled sides after this pass: 12W-5L across 17.</t>
+          <t>[WORKED] Coventry @ Arsenal, EPL opener (3:00 PM ET Fri, Emirates): NOT FILLED - best named-book price all day was DK -475 (1.211); the 1.224 trigger never printed (FanDuel closed -550). Arsenal won 3-0: a would-have-won that never offered the price. The extreme-favorite demotion was correct: the market's ceiling sat below our bar all day.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] Jets @ Steelers, NFL preseason Wk 2 (7:00 PM ET Fri, Acrisure): FILL CONDITION MET AT NAMED BOOKS - AND WON. The 'drift toward PIT' we flagged at ship was the OPENER (PIT -3, Jets 2.47); named books held Jets above the 1.804 trigger all day and DK closed Jets -122 (1.82). Jets won 17-0. Paper grade at the 1.804 floor: raw CLV -0.9%, no-vig -4.8% - roughly flat, because the conservative floor sits at the close; anything nearer the open was strongly positive. Second paper fill in ledger history; both cashed. Lesson: our unnamed-book preseason snapshot (1.70) was the soft side of a market that was never there - named-book conditions turn soft snapshots into real prices. Stake 0 - backup order, user bets headline only.</t>
+          <t>[WORKED] Coventry @ Arsenal, same match - total 2.5: NOT FILLED - Over 2.5 closed -176/-181 (1.552-1.568); the 1.662 trigger never evidenced. It landed (3 goals) and SportsLine's 64% graded RIGHT on its first EPL outing - a model note for the file, priced away by the market. Never-filled sides after this pass: 12W-5L across 17.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] Atlas @ Cruz Azul, Liga MX J5 (11:00 PM ET Sat, Estadio Banorte/Azteca): STOOD DOWN PER DRIFT-CANCEL - and the rule saved the ticket. The board drifted from Caliente -205/Codere -200 THROUGH the 1.569 trigger (a Betway 1.62 shows on Aug-22 comparison pages, timing unverified; Dimers' -190 board does NOT clear). The slip's printed rule covers exactly this: a drift-through is a changed premise - re-price and stand down. The drift was the market fading Cruz Azul, and Cruz Azul lost 0-2 at home. CONDITIONAL SAVE #7 (the drift-taker loses). FILL ORACLE OPEN: if you actually took 1.62, report it and I regrade as a loss at your stake (Braves precedent). Drift-throughs are now 0-for-3 as bets (Liberty, Braves, this).</t>
+          <t>[WORKED] Jets @ Steelers, NFL preseason Wk 2 (7:00 PM ET Fri, Acrisure): FILL CONDITION MET AT NAMED BOOKS - AND WON. The 'drift toward PIT' we flagged at ship was the OPENER (PIT -3, Jets 2.47); named books held Jets above the 1.804 trigger all day and DK closed Jets -122 (1.82). Jets won 17-0. Paper grade at the 1.804 floor: raw CLV -0.9%, no-vig -4.8% - roughly flat, because the conservative floor sits at the close; anything nearer the open was strongly positive. Second paper fill in ledger history; both cashed. Lesson: our unnamed-book preseason snapshot (1.70) was the soft side of a market that was never there - named-book conditions turn soft snapshots into real prices. Stake 0 - backup order, user bets headline only.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] Hernandez vs Rodrigues, UFC FN Sacramento main event (~10:15 PM ET walk): NOT FILLED - the first UFC order's line steamed the wrong way all week (DK -166 -&gt; Hard Rock -185 -&gt; DK -198 close); -145 never existed. COUNTERFACTUAL SAVE #6: Rodrigues won the fight by UD at +164 - a fill would have lost. The steam was information, again.</t>
+          <t>[WORKED] Atlas @ Cruz Azul, Liga MX J5 (11:00 PM ET Sat, Estadio Banorte/Azteca): STOOD DOWN PER DRIFT-CANCEL - and the rule saved the ticket. The board drifted from Caliente -205/Codere -200 THROUGH the 1.569 trigger (a Betway 1.62 shows on Aug-22 comparison pages, timing unverified; Dimers' -190 board does NOT clear). The slip's printed rule covers exactly this: a drift-through is a changed premise - re-price and stand down. The drift was the market fading Cruz Azul, and Cruz Azul lost 0-2 at home. CONDITIONAL SAVE #7 (the drift-taker loses). FILL ORACLE OPEN: if you actually took 1.62, report it and I regrade as a loss at your stake (Braves precedent). Drift-throughs are now 0-for-3 as bets (Liberty, Braves, this).</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] Hamilton @ Toronto, CFL Wk 12 (7:00 PM ET Sat, BMO Field): NOT FILLED - no named book ever better than -225 vs the -187 trigger (the unattributed -218 we demoted was close to true). Argos won 39-20, a would-have-won at a price that never existed. Note: the WEATHER CLAUSE actually TRIGGERED (thunderstorm-delayed start) - had anything filled, the printed clause voided it anyway. Clause class: 3-for-3 firing correctly when conditions hit.</t>
+          <t>[WORKED] Hernandez vs Rodrigues, UFC FN Sacramento main event (~10:15 PM ET walk): NOT FILLED - the first UFC order's line steamed the wrong way all week (DK -166 -&gt; Hard Rock -185 -&gt; DK -198 close); -145 never existed. COUNTERFACTUAL SAVE #6: Rodrigues won the fight by UD at +164 - a fill would have lost. The steam was information, again.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] Boca Juniors @ Racing Club, Clausura fecha 6 (8:30 PM ET Sun, El Cilindro): NOT FILLED - no named book ever printed Boca near +177 (best found: bplay 2.60, Betsson 2.55, bet365 DNB 1.62 implying ~2.4-2.6); the trigger sat ~8% above the whole named market. COUNTERFACTUAL SAVE #7: the match ended 1-1, so any filled 90-minute ticket loses - and the draw-heavy H2H that set the high bar was exactly the risk that landed. Never-filled orders' sides now 14W-8L across 22.</t>
+          <t>[WORKED] Hamilton @ Toronto, CFL Wk 12 (7:00 PM ET Sat, BMO Field): NOT FILLED - no named book ever better than -225 vs the -187 trigger (the unattributed -218 we demoted was close to true). Argos won 39-20, a would-have-won at a price that never existed. Note: the WEATHER CLAUSE actually TRIGGERED (thunderstorm-delayed start) - had anything filled, the printed clause voided it anyway. Clause class: 3-for-3 firing correctly when conditions hit.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] PIT @ SD (9:40 PM ET Mon, Petco; PITCHERS: Ashcraft vs Robbie Ray): WON - the first tier bet cashes. PIT 3-2 in 12; $35 at 2.00 returns $70 (+$35 at the reference stake - report your actual book/price/stake and I restate real P&amp;L). Ashcraft/Ray premise held; bet365 +100 documented at the latest pre-game snapshot. CLV at the split close: raw +4.8% vs the -110/-110 consensus, no-vig +0.0% (book range -3.3% to +1.3%) - we took the best price on the board and the market ended where we bet it. TIER SCOREBOARD: 1 settled, 1-0, mean no-vig CLV ~0.0%; 14 more to the pre-registered rollback checkpoint.</t>
+          <t>[WORKED] Boca Juniors @ Racing Club, Clausura fecha 6 (8:30 PM ET Sun, El Cilindro): NOT FILLED - no named book ever printed Boca near +177 (best found: bplay 2.60, Betsson 2.55, bet365 DNB 1.62 implying ~2.4-2.6); the trigger sat ~8% above the whole named market. COUNTERFACTUAL SAVE #7: the match ended 1-1, so any filled 90-minute ticket loses - and the draw-heavy H2H that set the high bar was exactly the risk that landed. Never-filled orders' sides now 14W-8L across 22.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] PHI @ SEA (9:40 PM ET Mon, T-Mobile Park; Wheeler vs Gilbert): STOOD DOWN PER DRIFT-CANCEL - SAVE #8. A named-book -108 print IS evidenced intraday (NBC/DK-network content), but it was a TRANSIENT CROSS: the board sat -115 below the trigger, touched -108, and closed back at -115/-118. Taxonomy now codified: a market STANDING above the trigger all day = legitimate fill (Jets precedent); a market that transiently CROSSES the trigger = drift-through, re-price and stand down (Liberty/Braves/Cruz Azul/this - drift-throughs now 0-for-4 as bets). PHI lost 2-9 (Wheeler 5-run 1st); a -108 fill was -1.6% no-vig CLV AND a full-stake loss. Fill oracle open: if you took -108, report it and I regrade.</t>
+          <t>[WORKED] PIT @ SD (9:40 PM ET Mon, Petco; PITCHERS: Ashcraft vs Robbie Ray): WON - the first tier bet cashes. PIT 3-2 in 12; $35 at 2.00 returns $70 (+$35 at the reference stake - report your actual book/price/stake and I restate real P&amp;L). Ashcraft/Ray premise held; bet365 +100 documented at the latest pre-game snapshot. CLV at the split close: raw +4.8% vs the -110/-110 consensus, no-vig +0.0% (book range -3.3% to +1.3%) - we took the best price on the board and the market ended where we bet it. TIER SCOREBOARD: 1 settled, 1-0, mean no-vig CLV ~0.0%; 14 more to the pre-registered rollback checkpoint.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] CHC @ AZ (9:40 PM ET Tue, Chase Field; Holmes vs Pfaadt): STOOD DOWN PER DRIFT-CANCEL - and this one is the rule's first counterfactual MISS. DK printed AZ +101 (&gt;= the 2.005 trigger) pre-game, but the board moved TOWARD the Cubs everywhere else (-105/-105 open -&gt; BetMGM -110s, SI CHC -112): a drift-through, not a standing price. Re-priced at the drifted number the blend gave -0.15% - below the model bar - so the stand-down was rule-correct. AZ then won 5-4 on a walk-off. Drift-throughs as hypothetical bets: 1-for-5 (Liberty, Braves, Cruz Azul, PHI lost; this won). The rule keeps its job on the aggregate; the miss is logged, not hidden.</t>
+          <t>[WORKED] PHI @ SEA (9:40 PM ET Mon, T-Mobile Park; Wheeler vs Gilbert): STOOD DOWN PER DRIFT-CANCEL - SAVE #8. A named-book -108 print IS evidenced intraday (NBC/DK-network content), but it was a TRANSIENT CROSS: the board sat -115 below the trigger, touched -108, and closed back at -115/-118. Taxonomy now codified: a market STANDING above the trigger all day = legitimate fill (Jets precedent); a market that transiently CROSSES the trigger = drift-through, re-price and stand down (Liberty/Braves/Cruz Azul/this - drift-throughs now 0-for-4 as bets). PHI lost 2-9 (Wheeler 5-run 1st); a -108 fill was -1.6% no-vig CLV AND a full-stake loss. Fill oracle open: if you took -108, report it and I regrade.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] WAS @ PHX (10:00 PM ET Tue, Footprint Center): NOT FILLED - the only -128 print was an unnamed aggregator leg; named books ran -130/-135. The fires-only-at-named-books condition held. Mystics won 94-84: a would-have-won at a price never verified to exist. Never-filled sides: 16W-9L across 26 after this card.</t>
+          <t>[WORKED] CHC @ AZ (9:40 PM ET Tue, Chase Field; Holmes vs Pfaadt): STOOD DOWN PER DRIFT-CANCEL - and this one is the rule's first counterfactual MISS. DK printed AZ +101 (&gt;= the 2.005 trigger) pre-game, but the board moved TOWARD the Cubs everywhere else (-105/-105 open -&gt; BetMGM -110s, SI CHC -112): a drift-through, not a standing price. Re-priced at the drifted number the blend gave -0.15% - below the model bar - so the stand-down was rule-correct. AZ then won 5-4 on a walk-off. Drift-throughs as hypothetical bets: 1-for-5 (Liberty, Braves, Cruz Azul, PHI lost; this won). The rule keeps its job on the aggregate; the miss is logged, not hidden.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] PIT @ SD (9:40 PM ET Tue, Petco; SKENES vs Michael King): FILLED AT A STANDING CROSS-BOOK PRICE - AND WON. BetMGM's own game blog quoted PIT +105 (2.05 &gt;= the 2.028 trigger) while the FanDuel anchor sat -104/-102: the Jets shape (standing-above, not a transient cross), so the fill is legitimate. PIT won 1-0 behind Skenes. Paper grade at the 2.028 floor: raw CLV +0.9%, no-vig -2.4%. numberFire's 55.8% lean graded RIGHT. Stake 0 - backup order, user bets headline only. TIER SCOREBOARD: 2 settled (Mon ticket + this), 2-0 on results, but no-vig CLV is Mon ~0.0% / this -2.4% - mean ~-1.2%, NEGATIVE. That is the pre-registered rollback metric: if it is still &lt;0 at 15 settled, both tiers revert to 2.5%. 13 to the checkpoint.</t>
+          <t>[WORKED] WAS @ PHX (10:00 PM ET Tue, Footprint Center): NOT FILLED - the only -128 print was an unnamed aggregator leg; named books ran -130/-135. The fires-only-at-named-books condition held. Mystics won 94-84: a would-have-won at a price never verified to exist. Never-filled sides: 16W-9L across 26 after this card.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] Brewers @ Mets, MLB (7:10 PM ET Wed, Citi Field): NOT FILLED - the trigger price is not evidenced as ever standing. Best named-book MIL price found anywhere pre-game: DraftKings -149 (1.671), four cents short of the -145 trigger; BetRivers held -165 and no Polymarket ask at 59c or lower surfaced. MIL won 8-1 - a would-have-won at a price that never existed (never-filled sides now ~17W-9L across 27). Footnote that matters: Dustin May exited after ONE PITCH (comebacker off the scapula). A fill would have survived the premise (he started), but the win would have been carried entirely by Gasser's relief work - the listed-pitcher clause is doing real risk work even on nights it technically holds.</t>
+          <t>[WORKED] PIT @ SD (9:40 PM ET Tue, Petco; SKENES vs Michael King): FILLED AT A STANDING CROSS-BOOK PRICE - AND WON. BetMGM's own game blog quoted PIT +105 (2.05 &gt;= the 2.028 trigger) while the FanDuel anchor sat -104/-102: the Jets shape (standing-above, not a transient cross), so the fill is legitimate. PIT won 1-0 behind Skenes. Paper grade at the 2.028 floor: raw CLV +0.9%, no-vig -2.4%. numberFire's 55.8% lean graded RIGHT. Stake 0 - backup order, user bets headline only. TIER SCOREBOARD: 2 settled (Mon ticket + this), 2-0 on results, but no-vig CLV is Mon ~0.0% / this -2.4% - mean ~-1.2%, NEGATIVE. That is the pre-registered rollback metric: if it is still &lt;0 at 15 settled, both tiers revert to 2.5%. 13 to the checkpoint.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] Toluca vs Austin FC, Leagues Cup QF (8:30 PM ET Wed, Harrison NJ - neutral): REFUSAL VALIDATED - and the conflict resolved toward the sportsbook, as our sharpness demotion assumes. An independent named pre-game trio surfaced post-hoc (Toluca -185 / +300 / +425) devigging to ~59.6% Toluca - 5 points from BetUS's 65%, 10 from Kalshi's 50c. Toluca won 2-0 IN THE 90 (Helinho pen 53', Diaz 90+7'; Austin down a man from 40'). One sample, but both the price check and the result say the exchange cents were the off number. The 15-point venue gap was real and unpriceable at bet time; refusing was the only correct position. Kept from the same card: Valkyries -909 (demoted) won by 25 - demotion cost nothing, as designed: it prices risk, not outcomes.</t>
+          <t>[WORKED] Brewers @ Mets, MLB (7:10 PM ET Wed, Citi Field): NOT FILLED - the trigger price is not evidenced as ever standing. Best named-book MIL price found anywhere pre-game: DraftKings -149 (1.671), four cents short of the -145 trigger; BetRivers held -165 and no Polymarket ask at 59c or lower surfaced. MIL won 8-1 - a would-have-won at a price that never existed (never-filled sides now ~17W-9L across 27). Footnote that matters: Dustin May exited after ONE PITCH (comebacker off the scapula). A fill would have survived the premise (he started), but the win would have been carried entirely by Gasser's relief work - the listed-pitcher clause is doing real risk work even on nights it technically holds.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] Alouettes @ Blue Bombers, CFL Wk 13 (8:30 PM ET Fri, Princess Auto Stadium, Winnipeg): WON 44-28 - the third tier ticket cashes, and this one BEAT THE CLOSE decisively: 26c entry vs a book close that held +240 (raw CLV +13.1%) and a no-vig fair of ~28.2% (no-vig CLV +2.7%) while the spread moved toward Montreal all day. $23 at 3.846 returned $88.46 (+$65.46 at the reference stake - report your actual venue/price/stake and I restate real P&amp;L; Polymarket's indexed print held WPG 26c). The Timbers stand-down line never triggered. TIER SCOREBOARD: 3 settled, 3-0, no-vig CLVs 0.0% / -2.4% / +2.7% (power-devig no-vig, same method as the engine - the raw +13.1% shrinks because power devig assigns most of a longshot pair's juice to the dog) - mean +0.1%, positive for the first time but barely; 12 to the rollback checkpoint.</t>
+          <t>[WORKED] Toluca vs Austin FC, Leagues Cup QF (8:30 PM ET Wed, Harrison NJ - neutral): REFUSAL VALIDATED - and the conflict resolved toward the sportsbook, as our sharpness demotion assumes. An independent named pre-game trio surfaced post-hoc (Toluca -185 / +300 / +425) devigging to ~59.6% Toluca - 5 points from BetUS's 65%, 10 from Kalshi's 50c. Toluca won 2-0 IN THE 90 (Helinho pen 53', Diaz 90+7'; Austin down a man from 40'). One sample, but both the price check and the result say the exchange cents were the off number. The 15-point venue gap was real and unpriceable at bet time; refusing was the only correct position. Kept from the same card: Valkyries -909 (demoted) won by 25 - demotion cost nothing, as designed: it prices risk, not outcomes.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] Red Sox @ Yankees, MLB (7:05 PM ET Fri, Yankee Stadium): NOT FILLED - no named book ever printed NYY -139 or better (evidenced range -148 to -173) and Polymarket stood at 59c (a Covers column even flagged taking NYY 'up to 59 cents' - consistent with our one-cent miss). NYY won 1-0: another would-have-won at a price that never existed. Never-filled sides ~18W-9L.</t>
+          <t>[WORKED] Alouettes @ Blue Bombers, CFL Wk 13 (8:30 PM ET Fri, Princess Auto Stadium, Winnipeg): WON 44-28 - the third tier ticket cashes, and this one BEAT THE CLOSE decisively: 26c entry vs a book close that held +240 (raw CLV +13.1%) and a no-vig fair of ~28.2% (no-vig CLV +2.7%) while the spread moved toward Montreal all day. $23 at 3.846 returned $88.46 (+$65.46 at the reference stake - report your actual venue/price/stake and I restate real P&amp;L; Polymarket's indexed print held WPG 26c). The Timbers stand-down line never triggered. TIER SCOREBOARD: 3 settled, 3-0, no-vig CLVs 0.0% / -2.4% / +2.7% (power-devig no-vig, same method as the engine - the raw +13.1% shrinks because power devig assigns most of a longshot pair's juice to the dog) - mean +0.1%, positive for the first time but barely; 12 to the rollback checkpoint.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] Orioles @ Athletics, MLB (9:40 PM ET Fri, Sutter Health Park, West Sacramento): NOT FILLED - AND THE CONDITION SAVED A LOSS. Aggregator picks-tables printed ATH +119/+120, but no NAMED book was ever behind those numbers and FanDuel (the named board) sat +100, under the +104 trigger. The fires-only-on-a-named-book-print condition held - and ATH LOST 3-4 in 10 innings, so an aggregator-print fill would have been a full-stake loser. This is the named-book condition's cleanest save yet (distinct from the 8 drift-cancel saves). Never-filled sides ~18W-10L across 29.</t>
+          <t>[WORKED] Red Sox @ Yankees, MLB (7:05 PM ET Fri, Yankee Stadium): NOT FILLED - no named book ever printed NYY -139 or better (evidenced range -148 to -173) and Polymarket stood at 59c (a Covers column even flagged taking NYY 'up to 59 cents' - consistent with our one-cent miss). NYY won 1-0: another would-have-won at a price that never existed. Never-filled sides ~18W-9L.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] Dodgers @ Tigers, MLB (6:40 PM ET Fri, Comerica Park) - the Skubal marquee: CONFLICT REFUSAL on the game everyone wanted: Skubal's revenge start. Two named books agree (BetRivers -225, FanDuel -215, ~67-69% LAD) while Polymarket sells LAD at 64c on $112K of volume - a 4-6 point venue fight whose best-price synthetic hold is NEGATIVE (-1.29%). The rule (degraded + negative cross-hold = unpriceable, never an arb) is 4-for-4 lifetime and was validated 48h ago by Toluca. POLICY QUESTION PRE-REGISTERED, not acted on: this shape differs from past conflicts - BOTH named books agree and only the exchange is off, and the candidate bet (LAD at PM 64c) is AT the outlier venue in the DIRECTION of the anchor consensus (+5.0% EV if the books are right, -0.6% if PM is right - positive under any mixture). Settle must record which venue was right here AND in the other three refusals (HOU@NYM, SEA@TOR, TEX@MIL); if the books-agree-exchange-off subtype keeps grading book-side-right, that is the ledger evidence a refinement needs. No parameter moves tonight (Walters rule). || SETTLED: the gap was REAL and the BOOKS were the better venue. FanDuel closed ~-215/+180 (no-vig LAD ~65.7%) vs Polymarket's 63-64c - a genuine ~2-point cross-venue disagreement that never converged. LAD won 2-1 behind Skubal (6 IP, 1 R in his Comerica return; under 7.5 cashed - our registered under lean RIGHT). Policy-question tally opens: books-agree-exchange-off subtype 1-0 books. A PM-side LAD bet at 64c would have won and carried positive CLV vs the book close - logged as the cost side of the refusal, per the honesty standard.</t>
+          <t>[WORKED] Orioles @ Athletics, MLB (9:40 PM ET Fri, Sutter Health Park, West Sacramento): NOT FILLED - AND THE CONDITION SAVED A LOSS. Aggregator picks-tables printed ATH +119/+120, but no NAMED book was ever behind those numbers and FanDuel (the named board) sat +100, under the +104 trigger. The fires-only-on-a-named-book-print condition held - and ATH LOST 3-4 in 10 innings, so an aggregator-print fill would have been a full-stake loser. This is the named-book condition's cleanest save yet (distinct from the 8 drift-cancel saves). Never-filled sides ~18W-10L across 29.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] HOU@NYM, SEA@TOR, TEX@MIL - three more venue conflicts, one card: Grouped refusal, engine-fired on all three: HOU@NYM (board HOU -128 vs Polymarket 51/50 pick'em on thin $59K - hold -0.70%), SEA@TOR (FanDuel -172 vs BET99 -155 one-sided - hold -0.45%; numberFire 53% TOR also far under the market), TEX@MIL (FanDuel -205 vs scoresandstats -181, 24 cents - hold -0.52%). Four refusals in one night is the dispersion mandate working as designed: hunting second venues finds gaps, and most gaps are somebody's bad quote, not value. Settle records the truth venue per game for the refusal-calibration ledger. || SETTLED, venue verdicts: TEX@MIL - FanDuel RIGHT (close clustered -190/-205; scoresandstats -181 was the stale outlier; MIL won 6-1). SEA@TOR - FanDuel RIGHT (close -161/-179 with FD dead-center; BET99 -155 sat outside the whole range; TOR won 8-1). HOU@NYM - THE EXCHANGE WAS RIGHT: the -128 board was stale and the market closed -105/-106, converging exactly to Polymarket's 51/50 (HOU won 3-1 - outcome noise; the close is the verdict). Running venue-calibration: named books 3, exchange 1 - and the exchange's win came against an unnamed consensus board, not against fresh named books. The sharpness hierarchy (named &gt; consensus &gt; exchange) survives the night.</t>
+          <t>[WORKED] Dodgers @ Tigers, MLB (6:40 PM ET Fri, Comerica Park) - the Skubal marquee: CONFLICT REFUSAL on the game everyone wanted: Skubal's revenge start. Two named books agree (BetRivers -225, FanDuel -215, ~67-69% LAD) while Polymarket sells LAD at 64c on $112K of volume - a 4-6 point venue fight whose best-price synthetic hold is NEGATIVE (-1.29%). The rule (degraded + negative cross-hold = unpriceable, never an arb) is 4-for-4 lifetime and was validated 48h ago by Toluca. POLICY QUESTION PRE-REGISTERED, not acted on: this shape differs from past conflicts - BOTH named books agree and only the exchange is off, and the candidate bet (LAD at PM 64c) is AT the outlier venue in the DIRECTION of the anchor consensus (+5.0% EV if the books are right, -0.6% if PM is right - positive under any mixture). Settle must record which venue was right here AND in the other three refusals (HOU@NYM, SEA@TOR, TEX@MIL); if the books-agree-exchange-off subtype keeps grading book-side-right, that is the ledger evidence a refinement needs. No parameter moves tonight (Walters rule). || SETTLED: the gap was REAL and the BOOKS were the better venue. FanDuel closed ~-215/+180 (no-vig LAD ~65.7%) vs Polymarket's 63-64c - a genuine ~2-point cross-venue disagreement that never converged. LAD won 2-1 behind Skubal (6 IP, 1 R in his Comerica return; under 7.5 cashed - our registered under lean RIGHT). Policy-question tally opens: books-agree-exchange-off subtype 1-0 books. A PM-side LAD bet at 64c would have won and carried positive CLV vs the book close - logged as the cost side of the refusal, per the honesty standard.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] Phillies @ D-backs, MLB (9:40 PM ET Mon, Chase Field): NOT FILLED BY ONE CENT - AND THE CLAUSE SAVED A LOSER AGAIN. Best named-book print all day: DraftKings +108 (2.08), one cent under the +109 trigger; FanDuel +100, consensus +105/+106; a lone '+109' mention appears in a snippet that simultaneously says 'best odds +103' - no verified standing print. AZ then LOST 1-2 (Nola out-dueled Pfaadt), so a fill would have graded L at ~flat CLV vs the +105/+106 close. That is the second consecutive card where the named-book/one-cent discipline refused a bet that loses (Fri ATH, Mon AZ). numberFire's 52.9% AZ graded WRONG. Never-filled sides ~18W-11L across 30 - the bars keep refusing the right ones lately.</t>
+          <t>[WORKED] HOU@NYM, SEA@TOR, TEX@MIL - three more venue conflicts, one card: Grouped refusal, engine-fired on all three: HOU@NYM (board HOU -128 vs Polymarket 51/50 pick'em on thin $59K - hold -0.70%), SEA@TOR (FanDuel -172 vs BET99 -155 one-sided - hold -0.45%; numberFire 53% TOR also far under the market), TEX@MIL (FanDuel -205 vs scoresandstats -181, 24 cents - hold -0.52%). Four refusals in one night is the dispersion mandate working as designed: hunting second venues finds gaps, and most gaps are somebody's bad quote, not value. Settle records the truth venue per game for the refusal-calibration ledger. || SETTLED, venue verdicts: TEX@MIL - FanDuel RIGHT (close clustered -190/-205; scoresandstats -181 was the stale outlier; MIL won 6-1). SEA@TOR - FanDuel RIGHT (close -161/-179 with FD dead-center; BET99 -155 sat outside the whole range; TOR won 8-1). HOU@NYM - THE EXCHANGE WAS RIGHT: the -128 board was stale and the market closed -105/-106, converging exactly to Polymarket's 51/50 (HOU won 3-1 - outcome noise; the close is the verdict). Running venue-calibration: named books 3, exchange 1 - and the exchange's win came against an unnamed consensus board, not against fresh named books. The sharpness hierarchy (named &gt; consensus &gt; exchange) survives the night.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] Giants @ Pirates, MLB (6:40 PM ET Tue, PNC Park) - Skenes vs Webb: NOT FILLED - no named book ever printed PIT -145 or better; the dated band was -158 (Athlon) to -162 (Predictem/DK -161). PIT then won 13-12 on a walk-off THROWING ERROR after blowing a six-run lead with Skenes shelled for 5 - a would-have-won that would have spent nine innings looking like a loser. The resting-order design priced the fill, not the outcome; a fill at the trigger would have carried ~+4% raw CLV vs the -161 close, which is exactly why the trigger sits where it sits. Never-filled sides ~19W-11L across 31.</t>
+          <t>[WORKED] Phillies @ D-backs, MLB (9:40 PM ET Mon, Chase Field): NOT FILLED BY ONE CENT - AND THE CLAUSE SAVED A LOSER AGAIN. Best named-book print all day: DraftKings +108 (2.08), one cent under the +109 trigger; FanDuel +100, consensus +105/+106; a lone '+109' mention appears in a snippet that simultaneously says 'best odds +103' - no verified standing print. AZ then LOST 1-2 (Nola out-dueled Pfaadt), so a fill would have graded L at ~flat CLV vs the +105/+106 close. That is the second consecutive card where the named-book/one-cent discipline refused a bet that loses (Fri ATH, Mon AZ). numberFire's 52.9% AZ graded WRONG. Never-filled sides ~18W-11L across 30 - the bars keep refusing the right ones lately.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] Marlins @ Royals, MLB (7:40 PM ET Tue, Kauffman Stadium): CONFLICT REFUSAL, engine-fired at -7.41% cross-hold: BetRivers prints KC -117 while YouWager prints MIA -160 - 50+ cents apart, the favorite FLIPS between boards. Per the post-phantom-anchor hierarchy (adopted after the MIL -196 grade), a conflict this size is encoded intact and refused, never resolved by hand - one of these boards is fiction and settle will record WHICH, feeding the calibration that already reads named-book &gt; exchange &gt; unnamed-article. DK splits (86% ML handle on KC) lean toward BetRivers being live, but handle is color, not truth. || SETTLED: KC closed the favorite at -117 (BetRivers) / -120 (DraftKings, sharps 66% bets / 88% dollars). The YouWager 'MIA -160' board was FICTION - a 40-cent inversion of the real market that appears only on that blog. Refusal validated on process; MIA won 6-3 as the +100 dog (outcome noise - the close is the verdict). Venue-truth ledger: named books 4, exchange 2, blog boards 0-for-3 this week.</t>
+          <t>[WORKED] Giants @ Pirates, MLB (6:40 PM ET Tue, PNC Park) - Skenes vs Webb: NOT FILLED - no named book ever printed PIT -145 or better; the dated band was -158 (Athlon) to -162 (Predictem/DK -161). PIT then won 13-12 on a walk-off THROWING ERROR after blowing a six-run lead with Skenes shelled for 5 - a would-have-won that would have spent nine innings looking like a loser. The resting-order design priced the fill, not the outcome; a fill at the trigger would have carried ~+4% raw CLV vs the -161 close, which is exactly why the trigger sits where it sits. Never-filled sides ~19W-11L across 31.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] Colorado @ Georgia Tech, CFB Week 1 (8:00 PM ET Thu, Bobby Dodd Stadium, ESPN): NOT FILLED BY THREE CENTS - AND THE SIDE WON 14-13. Best named print all day: DraftKings +220 (3.20) against the +223 (3.23) trigger; FanDuel and bet365 +205; the unnamed +240 was the pre-ship opener. The market moved TOWARD Colorado all day on sharp money (DK: 10% of tickets / 63% of handle), which is why the trigger - set 1.5% above a blended fair that weights the market 0.85 - drifted out of reach instead of into it. Colorado won on a TD with 0:42 left and a blocked field goal. The ledger's first CFB order: a missed winner, honestly logged. Never-filled sides ~20W-11L across 32.</t>
+          <t>[WORKED] Marlins @ Royals, MLB (7:40 PM ET Tue, Kauffman Stadium): CONFLICT REFUSAL, engine-fired at -7.41% cross-hold: BetRivers prints KC -117 while YouWager prints MIA -160 - 50+ cents apart, the favorite FLIPS between boards. Per the post-phantom-anchor hierarchy (adopted after the MIL -196 grade), a conflict this size is encoded intact and refused, never resolved by hand - one of these boards is fiction and settle will record WHICH, feeding the calibration that already reads named-book &gt; exchange &gt; unnamed-article. DK splits (86% ML handle on KC) lean toward BetRivers being live, but handle is color, not truth. || SETTLED: KC closed the favorite at -117 (BetRivers) / -120 (DraftKings, sharps 66% bets / 88% dollars). The YouWager 'MIA -160' board was FICTION - a 40-cent inversion of the real market that appears only on that blog. Refusal validated on process; MIA won 6-3 as the +100 dog (outcome noise - the close is the verdict). Venue-truth ledger: named books 4, exchange 2, blog boards 0-for-3 this week.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] Pachuca @ FC Juarez, Liga MX Apertura J7 (11:00 PM ET Fri, Estadio Olimpico Benito Juarez): WON - Pachuca 2-0 at Juarez, the fourth tier ticket and the second sourced from an exchange. $104 at 2.174 returns $226.10 (+$122.10 at the reference stake - report your actual venue, price and size and I restate real P&amp;L). SETTLEMENT PREMISE CONFIRMED INDEPENDENTLY: Robinhood's listing of the same contract words it '90 minutes plus stoppage, excluding extra time and penalties' - exactly the market we priced, and both goals came in regulation, so there was no ambiguity. The 46c ask was corroborated as a real quoted price by a second source ('Kalshi has Pachuca at 46%'), though NO volume or depth figure is indexed anywhere - fill size remains unverified by anything but your own report. CLV IS GENUINELY AMBIGUOUS and is recorded conservatively. Raw +11.4%% against the ESPN BET board we anchored on, which re-indexed unchanged at 1.952. But that page serves a single untimestamped snapshot, and a second dated board had Pachuca LENGTHENING to +102 while Juarez shortened - implying a closing Pachuca near 45.8%% against ESPN BET's 49.2%%. The honest bracket on no-vig CLV is -0.4%% to +7.0%%; clv_novig is set to 0.0 at the conservative end BECAUSE this figure feeds the pre-registered rollback metric, and a metric that can retire a policy should never be flattered. TIER SCOREBOARD: 4 settled, 4-0 on results, mean no-vig CLV ~+0.1%% - still barely above zero after four bets; 11 to the checkpoint. This ticket is money in hand and a neutral process verdict: it is NOT evidence the Liga MX blend works.</t>
+          <t>[WORKED] Colorado @ Georgia Tech, CFB Week 1 (8:00 PM ET Thu, Bobby Dodd Stadium, ESPN): NOT FILLED BY THREE CENTS - AND THE SIDE WON 14-13. Best named print all day: DraftKings +220 (3.20) against the +223 (3.23) trigger; FanDuel and bet365 +205; the unnamed +240 was the pre-ship opener. The market moved TOWARD Colorado all day on sharp money (DK: 10% of tickets / 63% of handle), which is why the trigger - set 1.5% above a blended fair that weights the market 0.85 - drifted out of reach instead of into it. Colorado won on a TD with 0:42 left and a blocked field goal. The ledger's first CFB order: a missed winner, honestly logged. Never-filled sides ~20W-11L across 32.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] Toledo @ Michigan State, CFB Week 1 (8:00 PM ET Fri, Spartan Stadium): CONFLICT REFUSAL, engine-fired at -5.25% best-price cross-venue hold. FanDuel's -420 devigs to ~77% Michigan State and KALSHI AGREES at 78c on $79K of volume - but POLYMARKET sits at 83c, five-plus points clear of both. Taking the cheap Toledo side at Polymarket's 17c against Kalshi's MSU 78c is the synthetic-arb shape that has graded wrong three times in this ledger. Note the asymmetry that makes this different from Wednesday's phantom-anchor inversion: there the lone outlier was an unnamed blog board and the exchange was right; here a NAMED book and an exchange agree and the other exchange is the outlier - which is exactly why the hierarchy says refuse rather than pick. Settle records which venue was right. Independent reason to stay away: SP+ has MSU by 13.8 and FPI by 5.4 - a two-touchdown model disagreement on a game with two first-time starting QBs under two new head coaches. || SETTLED - VALIDATED ON PROCESS AND OUTCOME. Michigan State won 30-20 (and did NOT cover -10.5), so the refused Toledo ticket would have LOST outright. The venue ranking against a ~77% closing consensus: FanDuel -420 was dead on (error ~0.0-0.7 points), KALSHI's 78c tracked it within a point, and POLYMARKET's 83c was six points off and NEVER CONVERGED - its market ranged 75-83% across $79K of volume, so the quote we saw sat at the extreme top of its own band. That is the unstable-cross-source signature the refusal rule exists to catch: the apparent six-point edge on Toledo at 17c was venue noise inside an eight-point band, not dispersion. Venue-truth ledger: named books 5, exchange 2. Polymarket stays demoted at 0.45 - nothing here argues otherwise.</t>
+          <t>[WORKED] Pachuca @ FC Juarez, Liga MX Apertura J7 (11:00 PM ET Fri, Estadio Olimpico Benito Juarez): WON - Pachuca 2-0 at Juarez, the fourth tier ticket and the second sourced from an exchange. $104 at 2.174 returns $226.10 (+$122.10 at the reference stake - report your actual venue, price and size and I restate real P&amp;L). SETTLEMENT PREMISE CONFIRMED INDEPENDENTLY: Robinhood's listing of the same contract words it '90 minutes plus stoppage, excluding extra time and penalties' - exactly the market we priced, and both goals came in regulation, so there was no ambiguity. The 46c ask was corroborated as a real quoted price by a second source ('Kalshi has Pachuca at 46%'), though NO volume or depth figure is indexed anywhere - fill size remains unverified by anything but your own report. CLV IS GENUINELY AMBIGUOUS and is recorded conservatively. Raw +11.4%% against the ESPN BET board we anchored on, which re-indexed unchanged at 1.952. But that page serves a single untimestamped snapshot, and a second dated board had Pachuca LENGTHENING to +102 while Juarez shortened - implying a closing Pachuca near 45.8%% against ESPN BET's 49.2%%. The honest bracket on no-vig CLV is -0.4%% to +7.0%%; clv_novig is set to 0.0 at the conservative end BECAUSE this figure feeds the pre-registered rollback metric, and a metric that can retire a policy should never be flattered. TIER SCOREBOARD: 4 settled, 4-0 on results, mean no-vig CLV ~+0.1%% - still barely above zero after four bets; 11 to the checkpoint. This ticket is money in hand and a neutral process verdict: it is NOT evidence the Liga MX blend works.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="21" t="inlineStr">
         <is>
-          <t>[WORKED] Patriots @ Seahawks, NFL Week 1 (8:20 PM ET Wed, Lumen Field): HEADLINE ORDER - dispersion tier (+1.0% bar; Kalshi at 0.45 sharpness sits below the 0.50 fair-line floor, so it is a shop venue, never a fair source). Fires at 37c or better (2.7027, +170). Blended fair 2.675 (37.38%); the model ensemble alone says 39.33%, so a 37c fill is +1.03% on the blend and +6.30% on the model. Best live prices: BetRivers +160 (a fair source, so it carries the +1.5% model-tier bar = 2.715 and misses), Kalshi 39c = 2.5641. TWO BINDING CLAUSES. (1) DRIFT-CANCEL WITH A NAMED TRIGGER: TreVeyon Henderson (NE RB) has not practiced since Aug 24 and his final designation was still outstanding at compile. If New England reaches 37c ON A HENDERSON-OUT HEADLINE, that is a drift, not a fill - the premise our fair was built on changed, the true probability moved down with the price, and we stand down and re-price. A 37c print on ordinary two-way flow with no news is a legitimate standing-above fill. Both graded drift-fills (Liberty Aug-3, Braves Aug-10) arrived exactly this way and both carried negative CLV. (2) BOOK-INTEGRITY FLOOR: the order is void if Kalshi's two legs sum to 100c or less (e.g. NE 36c against SEA 64c). Our own conflict rule refuses a zero/negative synthetic hold on a degraded anchor, and an exchange showing one is showing a stale side, not a gift. Verified at compile: NE 39c + SEA 63c = 102c. PREMISES HELD AT COMPILE: Maye and Darnold both entirely absent from the injury report; NE C Ben Brown OUT. $15 at quarter-Kelly if filled at 37c (returns $41); ~$54 at 36c. || CANCELLED Wed 2026-09-09 12:01Z (8:01 AM ET, ~12h pre-kickoff), on the fallback wake. THE NAMED TRIGGER FIRED: TreVeyon Henderson was RULED OUT on New England's final injury report, released Tuesday Sep 8 - the exact condition clause (1) was written against. Market state at cancellation: Kalshi SEA 63c / NE 38c (sum 101c, so the book-integrity floor in clause (2) held). TWO SEPARATE FACTS, and they matter independently. FIRST: the order never filled on its own terms - 38c never reached the 37c trigger, so this is a no-fill regardless of the premise. SECOND: the market moved one cent IN OUR FAVOUR (39c -&gt; 38c, i.e. New England got cheaper), and that is exactly the trap the clause exists to catch - the price improved BECAUSE the true probability fell, not because value appeared. Had the drift carried one more cent to 37c we would have been handed a trigger print on a side whose premise had just deteriorated, which is the shape of both graded drift-fills (Liberty Aug-3, Braves Aug-10) that carried negative CLV. Standing the order down rather than leaving a resting trigger we would not honour. NOT RE-PRICED: a fresh fair would need a new compile, and this is a fallback wake, not a GO. At the compile fair the 38c price is -1.63% on the blend (+3.50% on the model alone), so nothing clears in any case.</t>
+          <t>[WORKED] Toledo @ Michigan State, CFB Week 1 (8:00 PM ET Fri, Spartan Stadium): CONFLICT REFUSAL, engine-fired at -5.25% best-price cross-venue hold. FanDuel's -420 devigs to ~77% Michigan State and KALSHI AGREES at 78c on $79K of volume - but POLYMARKET sits at 83c, five-plus points clear of both. Taking the cheap Toledo side at Polymarket's 17c against Kalshi's MSU 78c is the synthetic-arb shape that has graded wrong three times in this ledger. Note the asymmetry that makes this different from Wednesday's phantom-anchor inversion: there the lone outlier was an unnamed blog board and the exchange was right; here a NAMED book and an exchange agree and the other exchange is the outlier - which is exactly why the hierarchy says refuse rather than pick. Settle records which venue was right. Independent reason to stay away: SP+ has MSU by 13.8 and FPI by 5.4 - a two-touchdown model disagreement on a game with two first-time starting QBs under two new head coaches. || SETTLED - VALIDATED ON PROCESS AND OUTCOME. Michigan State won 30-20 (and did NOT cover -10.5), so the refused Toledo ticket would have LOST outright. The venue ranking against a ~77% closing consensus: FanDuel -420 was dead on (error ~0.0-0.7 points), KALSHI's 78c tracked it within a point, and POLYMARKET's 83c was six points off and NEVER CONVERGED - its market ranged 75-83% across $79K of volume, so the quote we saw sat at the extreme top of its own band. That is the unstable-cross-source signature the refusal rule exists to catch: the apparent six-point edge on Toledo at 17c was venue noise inside an eight-point band, not dispersion. Venue-truth ledger: named books 5, exchange 2. Polymarket stays demoted at 0.45 - nothing here argues otherwise.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="21" t="inlineStr">
         <is>
-          <t>[DIDN'T] CHC @ STL: Cashed on variance: close (CHC +100/STL -120, sharp money on STL) says the edge was not there. Fair missed the no-vig close by 3.7pts on a source-conflict market -&gt; conflict-refusal rule shipped.</t>
+          <t>[WORKED] Patriots @ Seahawks, NFL Week 1 - total 44.5: DECLINED READ, registered so it can be graded. Forecast for the 5:20-8:30 PM PT window at open-air Lumen: 20-30 mph gusts across the Puget Sound lowlands strengthening into the evening, plus moderate-to-heavy rain. That is a real under thesis and it is the most confident qualitative statement on this card. It is NOT BET for three independent reasons, any one of which is sufficient: totals never headline (standing rule); FanDuel and BookmakersReview both sit 44.5 -110/-110 with zero cross-venue dispersion, so there is no venue to buy it at; and we carry no calibrated weather model, so any probability we asserted would be invented. The ESPN listing's 45.5 would be the number to buy under if it were real, but it is one-sided and undated. Settle should record whether the game went under 44.5 - if this read keeps grading right while unpriced, that is evidence for building a weather layer, which is a parameter change and needs ledger evidence first. || SETTLED 2026-09-10. THE UNDER CASHED BY 21.5 POINTS - 23 total against 44.5 - AND THE THESIS WAS WRONG. The forecast 20-30 mph gusts and heavy rain NEVER MATERIALIZED: actual conditions were winds under 6 mph, gusts topping out at 9, and zero precipitation, with DK Network stating flatly that weather had no impact on the game. The 23 points came from defense and turnovers - three fourth-quarter New England interceptions and a Seattle offense that was shut out in the first half after losing Darnold on the opening drive. So a bet placed on our stated reasoning would have won money for a reason that did not happen. THIS IS EVIDENCE AGAINST BUILDING A WEATHER LAYER, NOT FOR ONE - the read was right and the model behind it was wrong, which is the single most misleading way for a thesis to grade. Declining stays correct on all three original grounds (totals never headline; both books at 44.5 -110/-110 with no venue to buy it; no calibrated weather model). Logged loudly so a future cycle does not cite 'the Lumen under' as support for weather modelling.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="21" t="inlineStr">
         <is>
-          <t>[DIDN'T] WSH @ ATL: VOID - PROCESS MISS (user report): the card shipped hours after this game's 1:35 PM ET first pitch. The container clock read Sunday evening; I overrode it because search snippets showed no Sunday finals - but a lagging search index is not pre-game proof. Order was never actionable; no bet placed, none should be. Original order terms preserved above for the record; outcome deliberately NOT graded (no hindsight grading of a void order).</t>
+          <t>[DIDN'T] CHC @ STL: Cashed on variance: close (CHC +100/STL -120, sharp money on STL) says the edge was not there. Fair missed the no-vig close by 3.7pts on a source-conflict market -&gt; conflict-refusal rule shipped.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="21" t="inlineStr">
         <is>
-          <t>[DIDN'T] BOS @ LAD (Sunday Night Baseball): VOID - cancelled at 7:03 PM ET with first pitch 7:20 PM ET: no time to re-verify the line, and every price on the card is a morning-stale snapshot. An unsupervisable order is not an order.</t>
+          <t>[DIDN'T] WSH @ ATL: VOID - PROCESS MISS (user report): the card shipped hours after this game's 1:35 PM ET first pitch. The container clock read Sunday evening; I overrode it because search snippets showed no Sunday finals - but a lagging search index is not pre-game proof. Order was never actionable; no bet placed, none should be. Original order terms preserved above for the record; outcome deliberately NOT graded (no hindsight grading of a void order).</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="21" t="inlineStr">
         <is>
-          <t>[DIDN'T] MIA @ NYM: VOID - shipped after the 1:40 PM ET first pitch (same process miss as the headline order). No bet placed, none should be.</t>
+          <t>[DIDN'T] BOS @ LAD (Sunday Night Baseball): VOID - cancelled at 7:03 PM ET with first pitch 7:20 PM ET: no time to re-verify the line, and every price on the card is a morning-stale snapshot. An unsupervisable order is not an order.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="21" t="inlineStr">
         <is>
+          <t>[DIDN'T] MIA @ NYM: VOID - shipped after the 1:40 PM ET first pitch (same process miss as the headline order). No bet placed, none should be.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="21" t="inlineStr">
+        <is>
+          <t>[DIDN'T] Patriots @ Seahawks, NFL Week 1 (8:20 PM ET Wed, Lumen Field): HEADLINE ORDER - dispersion tier (+1.0% bar; Kalshi at 0.45 sharpness sits below the 0.50 fair-line floor, so it is a shop venue, never a fair source). Fires at 37c or better (2.7027, +170). Blended fair 2.675 (37.38%); the model ensemble alone says 39.33%, so a 37c fill is +1.03% on the blend and +6.30% on the model. Best live prices: BetRivers +160 (a fair source, so it carries the +1.5% model-tier bar = 2.715 and misses), Kalshi 39c = 2.5641. TWO BINDING CLAUSES. (1) DRIFT-CANCEL WITH A NAMED TRIGGER: TreVeyon Henderson (NE RB) has not practiced since Aug 24 and his final designation was still outstanding at compile. If New England reaches 37c ON A HENDERSON-OUT HEADLINE, that is a drift, not a fill - the premise our fair was built on changed, the true probability moved down with the price, and we stand down and re-price. A 37c print on ordinary two-way flow with no news is a legitimate standing-above fill. Both graded drift-fills (Liberty Aug-3, Braves Aug-10) arrived exactly this way and both carried negative CLV. (2) BOOK-INTEGRITY FLOOR: the order is void if Kalshi's two legs sum to 100c or less (e.g. NE 36c against SEA 64c). Our own conflict rule refuses a zero/negative synthetic hold on a degraded anchor, and an exchange showing one is showing a stale side, not a gift. Verified at compile: NE 39c + SEA 63c = 102c. PREMISES HELD AT COMPILE: Maye and Darnold both entirely absent from the injury report; NE C Ben Brown OUT. $15 at quarter-Kelly if filled at 37c (returns $41); ~$54 at 36c. || CANCELLED Wed 2026-09-09 12:01Z (8:01 AM ET, ~12h pre-kickoff), on the fallback wake. THE NAMED TRIGGER FIRED: TreVeyon Henderson was RULED OUT on New England's final injury report, released Tuesday Sep 8 - the exact condition clause (1) was written against. Market state at cancellation: Kalshi SEA 63c / NE 38c (sum 101c, so the book-integrity floor in clause (2) held). TWO SEPARATE FACTS, and they matter independently. FIRST: the order never filled on its own terms - 38c never reached the 37c trigger, so this is a no-fill regardless of the premise. SECOND: the market moved one cent IN OUR FAVOUR (39c -&gt; 38c, i.e. New England got cheaper), and that is exactly the trap the clause exists to catch - the price improved BECAUSE the true probability fell, not because value appeared. Had the drift carried one more cent to 37c we would have been handed a trigger print on a side whose premise had just deteriorated, which is the shape of both graded drift-fills (Liberty Aug-3, Braves Aug-10) that carried negative CLV. Standing the order down rather than leaving a resting trigger we would not honour. NOT RE-PRICED: a fresh fair would need a new compile, and this is a fallback wake, not a GO. At the compile fair the 38c price is -1.63% on the blend (+3.50% on the model alone), so nothing clears in any case. || SETTLED 2026-09-10. THREE FACTS, AND THEY DO NOT AGREE - recording all three. (1) NEVER FILLABLE. Kalshi's book sat 62 bid / 63 ask on Seattle all week, which is NE 37 BID / 38 ASK. Our 37c order was a bid joining the queue, not a takeable offer, and no source documents New England ever offered below 38c. So this was a no-fill on mechanics regardless of the cancel. (2) IT WOULD HAVE LOST. New England lost outright 13-10, so any fill loses the $15 stake. (3) AND YET IT GRADES AS A PROCESS MISS BY OUR OWN STANDARD. The close devigs to NE 0.3895; at 37c that is +5.28% no-vig CLV - by a wide margin the best CLV any order in this ledger has carried, against five prior fills that were ALL negative. Our doctrine says CLV, not P&amp;L, is the verdict. So: the price was right and we talked ourselves out of it. THE REASONING THAT FAILED: the drift-cancel clause assumed that if New England got cheaper after Henderson was ruled out, the price improved BECAUSE the true probability fell. That inference was testable and it was FALSE. The market moved toward New England all week - spread 3.5 -&gt; 3, DK ML -175 -&gt; -170 - which is precisely the convergence our own football module predicted when it devigged the spread to 3.29. We wrote a clause against news and it fired on a market correction our own model had already called. HYPOTHESIS PRE-REGISTERED, NOT ADOPTED (Walters rule, n=1): the drift-cancel test needs a second question - is the price moving AWAY from our model's number (real premise decay, stand down) or TOWARD it (the market agreeing with us, which is the opposite of a reason to cancel)? Needs more graded cases before it changes anything.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="21" t="inlineStr">
+        <is>
           <t>[DIDN'T] Calibration: flagged-source fair lines (conflict / date trap / low-confidence close) missed the no-vig close by 4.86 pts on average vs 1.92 pts for clean sources — source hygiene IS calibration.</t>
         </is>
       </c>
     </row>
-    <row r="99">
-      <c r="A99" s="22" t="inlineStr">
+    <row r="101">
+      <c r="A101" s="22" t="inlineStr">
         <is>
           <t>Source: data/track_record.json (SharpOds ledger); regenerated by `sharpods-tracker`. Assumption: closing lines are best-available day-of published numbers, not exchange-verified closing ticks.</t>
         </is>

</xml_diff>

<commit_message>
Regenerate tracker through the full Sep 9 settle
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Epz958ydWx4TMSQvnKeiSm
</commit_message>
<xml_diff>
--- a/data/tracker.xlsx
+++ b/data/tracker.xlsx
@@ -4692,7 +4692,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I229"/>
+  <dimension ref="A1:I230"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -13412,6 +13412,44 @@
         <v/>
       </c>
       <c r="I229" s="2" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B230" s="2" t="inlineStr">
+        <is>
+          <t>nfl-2026-09-10-sf-lar</t>
+        </is>
+      </c>
+      <c r="C230" s="8" t="n">
+        <v>0.6347</v>
+      </c>
+      <c r="D230" s="8" t="n">
+        <v>0.6478</v>
+      </c>
+      <c r="E230" s="9">
+        <f>ABS(C230-D230)*100</f>
+        <v/>
+      </c>
+      <c r="F230" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G230" s="10">
+        <f>(C230-F230)^2</f>
+        <v/>
+      </c>
+      <c r="H230" s="10">
+        <f>(D230-F230)^2</f>
+        <v/>
+      </c>
+      <c r="I230" s="2" t="inlineStr">
         <is>
           <t>clean</t>
         </is>

</xml_diff>